<commit_message>
Rework rebirth cycle bonus into a refund multiplier, not a stat bonus
Replaces the earlier all-stat multiplicative bonus with a refund-only
design: accumulated cycle points now scale how much currency you get
back on rebirth (capped by MaxRefundMultiplier), and no longer touch
in-run stats or currency gain at all. Points this rebirth earns apply
starting next rebirth, not to their own refund. Adds RefundBonusPerPoint
and MaxRefundMultiplier to RebirthTable, repurposes the former
"all-stat bonus" StringTable label as "refund multiplier", and expands
the rebirth modal to show base-to-actual refund amounts per currency.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -603,7 +603,7 @@
     <t>BonusBase</t>
   </si>
   <si>
-    <t>회차 보너스 포인트 공식의 기준 계수. 포인트 = floor(BonusBase × 도달스테이지^BonusExponent)</t>
+    <t>회차 보너스 포인트 공식의 기준 계수. 포인트 = BonusBase × 도달스테이지^BonusExponent (소수점 유지, 최소 스테이지 제한 없음)</t>
   </si>
   <si>
     <t/>
@@ -618,22 +618,22 @@
     <t>회차 보너스 포인트 공식에서 도달 스테이지에 적용하는 지수</t>
   </si>
   <si>
-    <t>포인트당 스탯 상승률</t>
-  </si>
-  <si>
-    <t>BonusPerPoint</t>
-  </si>
-  <si>
-    <t>누적 보너스 포인트 1당 전 스탯에 곱연산으로 붙는 상승률(%). 전 스탯 보너스율 = 누적 포인트 × 이 값</t>
-  </si>
-  <si>
-    <t>보너스 최소 스테이지</t>
-  </si>
-  <si>
-    <t>MinStageForBonus</t>
-  </si>
-  <si>
-    <t>리버스 시점의 도달 스테이지가 이 값 미만이면 보너스 포인트를 얻지 못함</t>
+    <t>포인트당 환급 증폭률</t>
+  </si>
+  <si>
+    <t>RefundBonusPerPoint</t>
+  </si>
+  <si>
+    <t>누적 보너스 포인트 1당 리버스 환급량에 곱연산으로 붙는 증폭률(%). 환급 배율 = 1 + (누적 포인트 × 이 값 / 100). 전투 중 재화 획득량/스탯에는 영향 없음</t>
+  </si>
+  <si>
+    <t>환급 배율 상한</t>
+  </si>
+  <si>
+    <t>MaxRefundMultiplier</t>
+  </si>
+  <si>
+    <t>환급 배율이 이 값을 넘지 않도록 제한</t>
   </si>
   <si>
     <t>보너스 설명</t>
@@ -1020,7 +1020,7 @@
     <t>스테이지/스탯/장비/숙련 초기화 + 소비 재화 전액 환급. 존재력 트리는 유지</t>
   </si>
   <si>
-    <t>포인트 = floor(1.0 × 도달스테이지^0.5), 10스테이지 미만이면 0. 전 스탯 보너스율(%) = 누적 포인트 × 1.0</t>
+    <t>포인트 = 1.0 × 도달스테이지^0.5 (소수점 유지, 최소 스테이지 제한 없음). 환급 배율 = 1 + (누적 포인트 × 1.0 / 100), 최대 5.0배. 전투 중 재화 획득량/스탯에는 영향 없음</t>
   </si>
   <si>
     <t>OfflineMaxHours</t>
@@ -1311,10 +1311,10 @@
     <t>PendingPoints</t>
   </si>
   <si>
-    <t>전 스탯 보너스</t>
-  </si>
-  <si>
-    <t>AllStatBonus</t>
+    <t>환급 배율</t>
+  </si>
+  <si>
+    <t>RefundMultiplier</t>
   </si>
   <si>
     <t>최고 도달 스테이지</t>
@@ -1327,7 +1327,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1367,10 +1367,17 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF7F6000"/>
+    </font>
+    <font>
       <b/>
       <color rgb="FFFFFF"/>
       <sz val="9"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <color rgb="1F3864"/>
@@ -1378,13 +1385,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF1F3864"/>
+    </font>
+    <font>
       <b/>
       <color rgb="1F3864"/>
       <sz val="9"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF1F3864"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1421,7 +1435,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="2F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5597"/>
       </patternFill>
     </fill>
     <fill>
@@ -1431,11 +1455,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="8EA9DB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8EA9DB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1473,11 +1507,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1487,6 +1536,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1503,14 +1558,26 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3519,22 +3586,22 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" s="3" t="s">
+      <c r="A93" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="B93" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="C93" s="3" t="s">
+      <c r="C93" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="D93" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E93" s="3" t="s">
+      <c r="D93" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E93" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="F93" s="3" t="s">
+      <c r="F93" s="4" t="s">
         <v>192</v>
       </c>
     </row>
@@ -3862,28 +3929,28 @@
     <col min="10" max="10" width="23" customWidth="1"/>
     <col min="11" max="11" width="17.3" customWidth="1"/>
     <col min="12" max="12" width="60" customWidth="1"/>
-    <col min="13" max="16" width="16" customWidth="1"/>
+    <col min="13" max="15" width="16" customWidth="1"/>
     <col min="17" max="17" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="10"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -3922,176 +3989,176 @@
       <c r="L2" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="12" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="N3" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="O3" s="10" t="s">
+      <c r="O3" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="P3" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q3" s="10" t="s">
+      <c r="P3" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q3" s="14" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="M4" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="N4" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="O4" s="11" t="s">
+      <c r="O4" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="P4" s="11" t="s">
+      <c r="P4" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="Q4" s="11" t="s">
+      <c r="Q4" s="16" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>35001</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="D5" s="7" t="b">
+      <c r="D5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="E5" s="7" t="b">
+      <c r="E5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="F5" s="7" t="b">
+      <c r="F5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="7" t="b">
+      <c r="G5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="H5" s="7" t="b">
+      <c r="H5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="I5" s="7" t="b">
+      <c r="I5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="J5" s="7" t="b">
+      <c r="J5" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="7" t="b">
+      <c r="K5" s="9" t="b">
         <v>1</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="M5" s="12">
+      <c r="M5" s="18">
         <v>1</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="18">
         <v>0.5</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="18">
         <v>1</v>
       </c>
-      <c r="P5" s="12">
-        <v>10</v>
+      <c r="P5" s="5">
+        <v>5</v>
       </c>
       <c r="Q5" s="3" t="s">
         <v>330</v>
@@ -4120,13 +4187,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4152,56 +4219,56 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>36001</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -4210,7 +4277,7 @@
       <c r="D5" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>8</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -4221,10 +4288,10 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>36002</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -4233,7 +4300,7 @@
       <c r="D6" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <v>1</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -4244,10 +4311,10 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>36003</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -4256,7 +4323,7 @@
       <c r="D7" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <v>0</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -4267,10 +4334,10 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>36004</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -4279,7 +4346,7 @@
       <c r="D8" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <v>0</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -4290,10 +4357,10 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>36005</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -4302,7 +4369,7 @@
       <c r="D9" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <v>0</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -4313,10 +4380,10 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="9">
         <v>6</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="9">
         <v>36006</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -4325,7 +4392,7 @@
       <c r="D10" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="9">
         <v>0</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -4336,10 +4403,10 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="9">
         <v>7</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="9">
         <v>36007</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -4348,7 +4415,7 @@
       <c r="D11" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="9">
         <v>0</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -4359,10 +4426,10 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="9">
         <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="9">
         <v>36008</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -4371,7 +4438,7 @@
       <c r="D12" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="9">
         <v>2</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -4402,11 +4469,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4426,44 +4493,44 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>40001</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -4477,10 +4544,10 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>40002</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -4494,10 +4561,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>40003</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -4511,10 +4578,10 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>40004</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -4528,10 +4595,10 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>40005</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -4545,10 +4612,10 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="9">
         <v>6</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="9">
         <v>40006</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -4562,10 +4629,10 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="9">
         <v>7</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="9">
         <v>40007</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -4579,10 +4646,10 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="9">
         <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="9">
         <v>40008</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -4596,10 +4663,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
-        <v>9</v>
-      </c>
-      <c r="B13" s="7">
+      <c r="A13" s="9">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
         <v>40009</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -4613,10 +4680,10 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
+      <c r="A14" s="9">
         <v>10</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="9">
         <v>40010</v>
       </c>
       <c r="C14" s="2" t="s">
@@ -4630,10 +4697,10 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
+      <c r="A15" s="9">
         <v>11</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="9">
         <v>40011</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -4647,10 +4714,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="7">
+      <c r="A16" s="9">
         <v>12</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="9">
         <v>40012</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -4664,10 +4731,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="7">
+      <c r="A17" s="9">
         <v>13</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="9">
         <v>40013</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -4681,10 +4748,10 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="7">
+      <c r="A18" s="9">
         <v>14</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="9">
         <v>40014</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -4698,10 +4765,10 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="7">
+      <c r="A19" s="9">
         <v>15</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="9">
         <v>40015</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -4715,10 +4782,10 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="7">
+      <c r="A20" s="9">
         <v>16</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="9">
         <v>40016</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -4732,10 +4799,10 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="7">
+      <c r="A21" s="9">
         <v>17</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="9">
         <v>40017</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -4749,10 +4816,10 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="7">
+      <c r="A22" s="9">
         <v>18</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22" s="9">
         <v>40018</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -4766,10 +4833,10 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="7">
+      <c r="A23" s="9">
         <v>19</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="9">
         <v>40019</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -4783,10 +4850,10 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="7">
+      <c r="A24" s="9">
         <v>20</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="9">
         <v>40020</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -4800,10 +4867,10 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="12">
+      <c r="A25" s="18">
         <v>21</v>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="18">
         <v>40021</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -4817,10 +4884,10 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="12">
+      <c r="A26" s="18">
         <v>22</v>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="18">
         <v>40022</v>
       </c>
       <c r="C26" s="3" t="s">
@@ -4834,10 +4901,10 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="12">
+      <c r="A27" s="18">
         <v>23</v>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="18">
         <v>40023</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -4851,10 +4918,10 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
+      <c r="A28" s="18">
         <v>24</v>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="18">
         <v>40024</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -4868,10 +4935,10 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="12">
+      <c r="A29" s="18">
         <v>25</v>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="18">
         <v>40025</v>
       </c>
       <c r="C29" s="3" t="s">
@@ -4885,10 +4952,10 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="12">
+      <c r="A30" s="18">
         <v>26</v>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="18">
         <v>40026</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -4902,10 +4969,10 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="12">
+      <c r="A31" s="18">
         <v>27</v>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="18">
         <v>40027</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -4919,10 +4986,10 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="12">
+      <c r="A32" s="18">
         <v>28</v>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="18">
         <v>40028</v>
       </c>
       <c r="C32" s="3" t="s">
@@ -4936,10 +5003,10 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="12">
+      <c r="A33" s="18">
         <v>29</v>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="18">
         <v>40029</v>
       </c>
       <c r="C33" s="3" t="s">
@@ -4953,10 +5020,10 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="12">
+      <c r="A34" s="18">
         <v>30</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="18">
         <v>40030</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -4970,10 +5037,10 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="12">
+      <c r="A35" s="18">
         <v>31</v>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="18">
         <v>40031</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -4987,10 +5054,10 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="12">
+      <c r="A36" s="18">
         <v>32</v>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="18">
         <v>40032</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -5004,10 +5071,10 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="12">
+      <c r="A37" s="18">
         <v>33</v>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="18">
         <v>40033</v>
       </c>
       <c r="C37" s="3" t="s">
@@ -5021,10 +5088,10 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="12">
+      <c r="A38" s="18">
         <v>34</v>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="18">
         <v>40034</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -5038,10 +5105,10 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="12">
+      <c r="A39" s="18">
         <v>35</v>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="18">
         <v>40035</v>
       </c>
       <c r="C39" s="3" t="s">
@@ -5055,10 +5122,10 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="12">
+      <c r="A40" s="18">
         <v>36</v>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="18">
         <v>40036</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -5072,10 +5139,10 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="12">
+      <c r="A41" s="18">
         <v>37</v>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="18">
         <v>40037</v>
       </c>
       <c r="C41" s="3" t="s">
@@ -5089,10 +5156,10 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="12">
+      <c r="A42" s="18">
         <v>38</v>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="18">
         <v>40038</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -5106,10 +5173,10 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="12">
+      <c r="A43" s="18">
         <v>39</v>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="18">
         <v>40039</v>
       </c>
       <c r="C43" s="3" t="s">
@@ -5123,10 +5190,10 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="12">
+      <c r="A44" s="18">
         <v>40</v>
       </c>
-      <c r="B44" s="12">
+      <c r="B44" s="18">
         <v>40040</v>
       </c>
       <c r="C44" s="3" t="s">
@@ -5140,10 +5207,10 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="12">
+      <c r="A45" s="18">
         <v>41</v>
       </c>
-      <c r="B45" s="12">
+      <c r="B45" s="18">
         <v>40041</v>
       </c>
       <c r="C45" s="3" t="s">
@@ -5157,10 +5224,10 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="12">
+      <c r="A46" s="18">
         <v>42</v>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="18">
         <v>40042</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -5174,10 +5241,10 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="12">
+      <c r="A47" s="18">
         <v>43</v>
       </c>
-      <c r="B47" s="12">
+      <c r="B47" s="18">
         <v>40043</v>
       </c>
       <c r="C47" s="3" t="s">
@@ -5191,10 +5258,10 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="12">
+      <c r="A48" s="18">
         <v>44</v>
       </c>
-      <c r="B48" s="12">
+      <c r="B48" s="18">
         <v>40044</v>
       </c>
       <c r="C48" s="3" t="s">
@@ -5208,10 +5275,10 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="12">
+      <c r="A49" s="18">
         <v>45</v>
       </c>
-      <c r="B49" s="12">
+      <c r="B49" s="18">
         <v>40045</v>
       </c>
       <c r="C49" s="3" t="s">
@@ -5225,10 +5292,10 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="12">
+      <c r="A50" s="18">
         <v>46</v>
       </c>
-      <c r="B50" s="12">
+      <c r="B50" s="18">
         <v>40046</v>
       </c>
       <c r="C50" s="3" t="s">
@@ -5242,10 +5309,10 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="12">
+      <c r="A51" s="18">
         <v>47</v>
       </c>
-      <c r="B51" s="12">
+      <c r="B51" s="18">
         <v>40047</v>
       </c>
       <c r="C51" s="3" t="s">
@@ -5259,10 +5326,10 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="12">
+      <c r="A52" s="18">
         <v>48</v>
       </c>
-      <c r="B52" s="12">
+      <c r="B52" s="18">
         <v>40048</v>
       </c>
       <c r="C52" s="3" t="s">
@@ -5276,10 +5343,10 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="12">
+      <c r="A53" s="18">
         <v>49</v>
       </c>
-      <c r="B53" s="12">
+      <c r="B53" s="18">
         <v>40049</v>
       </c>
       <c r="C53" s="3" t="s">
@@ -5293,10 +5360,10 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="12">
+      <c r="A54" s="18">
         <v>50</v>
       </c>
-      <c r="B54" s="12">
+      <c r="B54" s="18">
         <v>40050</v>
       </c>
       <c r="C54" s="3" t="s">
@@ -5310,10 +5377,10 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="12">
+      <c r="A55" s="18">
         <v>51</v>
       </c>
-      <c r="B55" s="12">
+      <c r="B55" s="18">
         <v>40051</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -5327,10 +5394,10 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="12">
+      <c r="A56" s="18">
         <v>52</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B56" s="18">
         <v>40052</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -5344,10 +5411,10 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="12">
+      <c r="A57" s="18">
         <v>53</v>
       </c>
-      <c r="B57" s="12">
+      <c r="B57" s="18">
         <v>40053</v>
       </c>
       <c r="C57" s="3" t="s">
@@ -5361,10 +5428,10 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="12">
+      <c r="A58" s="18">
         <v>54</v>
       </c>
-      <c r="B58" s="12">
+      <c r="B58" s="18">
         <v>40054</v>
       </c>
       <c r="C58" s="3" t="s">
@@ -5749,22 +5816,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -5811,970 +5878,970 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="M3" s="5" t="s">
+      <c r="H3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="7" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="8" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>10001</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>20</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>3</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="9">
         <v>5</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="9">
         <v>5</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="9">
         <v>2</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="9">
         <v>1</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="9">
         <v>0</v>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="9">
         <v>1.15</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>10002</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="9">
         <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <v>350</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <v>16</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="9">
         <v>1</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="9">
         <v>33</v>
       </c>
-      <c r="J6" s="7">
-        <v>9</v>
-      </c>
-      <c r="K6" s="7">
+      <c r="J6" s="9">
+        <v>9</v>
+      </c>
+      <c r="K6" s="9">
         <v>2</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="9">
         <v>5</v>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="9">
         <v>1.15</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>10003</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="9">
         <v>2</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="9">
         <v>80</v>
       </c>
-      <c r="G7" s="7">
-        <v>9</v>
-      </c>
-      <c r="H7" s="7">
+      <c r="G7" s="9">
+        <v>9</v>
+      </c>
+      <c r="H7" s="9">
         <v>5</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="9">
         <v>12</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="9">
         <v>4</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="9">
         <v>1</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="9">
         <v>0</v>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="9">
         <v>1.15</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>10004</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="9">
         <v>2</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="9">
         <v>1420</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <v>50</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="9">
         <v>1</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="9">
         <v>90</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <v>24</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="9">
         <v>4</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="9">
         <v>5</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="9">
         <v>1.15</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>10005</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="9">
         <v>3</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="9">
         <v>327</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="9">
         <v>28</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="9">
         <v>5</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="9">
         <v>33</v>
       </c>
-      <c r="J9" s="7">
-        <v>9</v>
-      </c>
-      <c r="K9" s="7">
+      <c r="J9" s="9">
+        <v>9</v>
+      </c>
+      <c r="K9" s="9">
         <v>2</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="9">
         <v>0</v>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="9">
         <v>1.15</v>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="9">
         <v>6</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="9">
         <v>10006</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="9">
         <v>3</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="9">
         <v>5755</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="9">
         <v>160</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="9">
         <v>1</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="9">
         <v>237</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="9">
         <v>54</v>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="9">
         <v>6</v>
       </c>
-      <c r="L10" s="7">
+      <c r="L10" s="9">
         <v>5</v>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="9">
         <v>1.15</v>
       </c>
-      <c r="N10" s="7">
+      <c r="N10" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="9">
         <v>7</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="9">
         <v>10007</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="9">
         <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11" s="9">
         <v>1324</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="9">
         <v>89</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="9">
         <v>5</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="9">
         <v>87</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="9">
         <v>20</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="9">
         <v>3</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="9">
         <v>0</v>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="9">
         <v>1.15</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="9">
         <v>8</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="9">
         <v>10008</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="9">
         <v>4</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="9">
         <v>23290</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="9">
         <v>498</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="9">
         <v>1</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="9">
         <v>615</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="9">
         <v>120</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="9">
         <v>8</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="9">
         <v>5</v>
       </c>
-      <c r="M12" s="7">
+      <c r="M12" s="9">
         <v>1.15</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
-        <v>9</v>
-      </c>
-      <c r="B13" s="7">
+      <c r="A13" s="9">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
         <v>10009</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="9">
         <v>5</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="9">
         <v>5357</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="9">
         <v>279</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="9">
         <v>5</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="9">
         <v>226</v>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="9">
         <v>43</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="9">
         <v>4</v>
       </c>
-      <c r="L13" s="7">
+      <c r="L13" s="9">
         <v>0</v>
       </c>
-      <c r="M13" s="7">
+      <c r="M13" s="9">
         <v>1.15</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="7">
+      <c r="A14" s="9">
         <v>10</v>
       </c>
-      <c r="B14" s="7">
+      <c r="B14" s="9">
         <v>10010</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="9">
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="9">
         <v>94230</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="9">
         <v>1548</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="9">
         <v>1</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="9">
         <v>1599</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="9">
         <v>258</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="9">
         <v>10</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L14" s="9">
         <v>5</v>
       </c>
-      <c r="M14" s="7">
+      <c r="M14" s="9">
         <v>1.15</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="7">
+      <c r="A15" s="9">
         <v>11</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="9">
         <v>10011</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="9">
         <v>6</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="9">
         <v>21673</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="9">
         <v>867</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="9">
         <v>5</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="9">
         <v>586</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="9">
         <v>93</v>
       </c>
-      <c r="K15" s="7">
+      <c r="K15" s="9">
         <v>5</v>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="9">
         <v>0</v>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="9">
         <v>1.15</v>
       </c>
-      <c r="N15" s="7">
+      <c r="N15" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="7">
+      <c r="A16" s="9">
         <v>12</v>
       </c>
-      <c r="B16" s="7">
+      <c r="B16" s="9">
         <v>10012</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="9">
         <v>6</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="9">
         <v>381215</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="9">
         <v>4808</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="9">
         <v>1</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="9">
         <v>4152</v>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="9">
         <v>561</v>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="9">
         <v>12</v>
       </c>
-      <c r="L16" s="7">
+      <c r="L16" s="9">
         <v>5</v>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="9">
         <v>1.15</v>
       </c>
-      <c r="N16" s="7">
+      <c r="N16" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="7">
+      <c r="A17" s="9">
         <v>13</v>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="9">
         <v>10013</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="9">
         <v>7</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="9">
         <v>87679</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="9">
         <v>2692</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="9">
         <v>5</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="9">
         <v>1522</v>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="9">
         <v>202</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="9">
         <v>6</v>
       </c>
-      <c r="L17" s="7">
+      <c r="L17" s="9">
         <v>0</v>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="9">
         <v>1.15</v>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="7">
+      <c r="A18" s="9">
         <v>14</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B18" s="9">
         <v>10014</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="9">
         <v>7</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18" s="9">
         <v>1542235</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="9">
         <v>14934</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="9">
         <v>1</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="9">
         <v>10767</v>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="9">
         <v>1212</v>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="9">
         <v>14</v>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="9">
         <v>5</v>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="9">
         <v>1.15</v>
       </c>
-      <c r="N18" s="7">
+      <c r="N18" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="7">
+      <c r="A19" s="9">
         <v>15</v>
       </c>
-      <c r="B19" s="7">
+      <c r="B19" s="9">
         <v>10015</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="9">
         <v>8</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="9">
         <v>354714</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="9">
         <v>8363</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="9">
         <v>5</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="9">
         <v>3948</v>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="9">
         <v>437</v>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="9">
         <v>7</v>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="9">
         <v>0</v>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="9">
         <v>1.15</v>
       </c>
-      <c r="N19" s="7">
+      <c r="N19" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="7">
+      <c r="A20" s="9">
         <v>16</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="9">
         <v>10016</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="9">
         <v>8</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20" s="9">
         <v>6239205</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="9">
         <v>46384</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="9">
         <v>1</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="9">
         <v>27930</v>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="9">
         <v>2619</v>
       </c>
-      <c r="K20" s="7">
+      <c r="K20" s="9">
         <v>16</v>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="9">
         <v>5</v>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="9">
         <v>1.15</v>
       </c>
-      <c r="N20" s="7">
+      <c r="N20" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="7">
+      <c r="A21" s="9">
         <v>17</v>
       </c>
-      <c r="B21" s="7">
+      <c r="B21" s="9">
         <v>10017</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="9">
         <v>9</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21" s="9">
         <v>1435017</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="9">
         <v>25975</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="9">
         <v>5</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="9">
         <v>10242</v>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="9">
         <v>943</v>
       </c>
-      <c r="K21" s="7">
+      <c r="K21" s="9">
         <v>8</v>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="9">
         <v>0</v>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="9">
         <v>1.15</v>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="7">
+      <c r="A22" s="9">
         <v>18</v>
       </c>
-      <c r="B22" s="7">
+      <c r="B22" s="9">
         <v>10018</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="9">
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="9">
         <v>25241070</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="9">
         <v>144062</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="9">
         <v>1</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="9">
         <v>72450</v>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="9">
         <v>5658</v>
       </c>
-      <c r="K22" s="7">
+      <c r="K22" s="9">
         <v>18</v>
       </c>
-      <c r="L22" s="7">
+      <c r="L22" s="9">
         <v>5</v>
       </c>
-      <c r="M22" s="7">
+      <c r="M22" s="9">
         <v>1.15</v>
       </c>
-      <c r="N22" s="7">
+      <c r="N22" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="7">
+      <c r="A23" s="9">
         <v>19</v>
       </c>
-      <c r="B23" s="7">
+      <c r="B23" s="9">
         <v>10019</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="9">
         <v>10</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="9">
         <v>5805446</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="9">
         <v>80675</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="9">
         <v>5</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="9">
         <v>26565</v>
       </c>
-      <c r="J23" s="7">
+      <c r="J23" s="9">
         <v>2037</v>
       </c>
-      <c r="K23" s="7">
-        <v>9</v>
-      </c>
-      <c r="L23" s="7">
+      <c r="K23" s="9">
+        <v>9</v>
+      </c>
+      <c r="L23" s="9">
         <v>0</v>
       </c>
-      <c r="M23" s="7">
+      <c r="M23" s="9">
         <v>1.15</v>
       </c>
-      <c r="N23" s="7">
+      <c r="N23" s="9">
         <v>1.1</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A24" s="7">
+      <c r="A24" s="9">
         <v>20</v>
       </c>
-      <c r="B24" s="7">
+      <c r="B24" s="9">
         <v>10020</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="9">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="9">
         <v>102114210</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="9">
         <v>447440</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="9">
         <v>1</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="9">
         <v>187917</v>
       </c>
-      <c r="J24" s="7">
+      <c r="J24" s="9">
         <v>12219</v>
       </c>
-      <c r="K24" s="7">
+      <c r="K24" s="9">
         <v>20</v>
       </c>
-      <c r="L24" s="7">
+      <c r="L24" s="9">
         <v>5</v>
       </c>
-      <c r="M24" s="7">
+      <c r="M24" s="9">
         <v>1.15</v>
       </c>
-      <c r="N24" s="7">
+      <c r="N24" s="9">
         <v>1.1</v>
       </c>
     </row>
@@ -6805,21 +6872,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -6857,80 +6924,80 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K3" s="5" t="s">
+      <c r="J3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>20001</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -6939,22 +7006,22 @@
       <c r="D5" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>40001</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>1</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>1</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="9">
         <v>8</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="9">
         <v>1.18</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="9">
         <v>9999</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -6962,10 +7029,10 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>20002</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -6974,22 +7041,22 @@
       <c r="D6" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <v>40002</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <v>1</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <v>1</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="9">
         <v>8</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="9">
         <v>1.18</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="9">
         <v>9999</v>
       </c>
       <c r="K6" s="2" t="s">
@@ -6997,10 +7064,10 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>20003</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -7009,22 +7076,22 @@
       <c r="D7" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <v>40003</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="9">
         <v>1</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <v>0.05</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="9">
         <v>8</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="9">
         <v>1.18</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="9">
         <v>9999</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -7032,10 +7099,10 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>20004</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -7044,22 +7111,22 @@
       <c r="D8" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <v>40004</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="9">
         <v>0</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <v>0.5</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="9">
         <v>8</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="9">
         <v>1.18</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <v>9999</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -7067,10 +7134,10 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>20005</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -7079,22 +7146,22 @@
       <c r="D9" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <v>40005</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="9">
         <v>150</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="9">
         <v>2</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="9">
         <v>8</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="9">
         <v>1.18</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="9">
         <v>9999</v>
       </c>
       <c r="K9" s="2" t="s">
@@ -7102,10 +7169,10 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="9">
         <v>6</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="9">
         <v>20006</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -7114,22 +7181,22 @@
       <c r="D10" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="9">
         <v>40006</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="9">
         <v>1</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="9">
         <v>0.02</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="9">
         <v>8</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="9">
         <v>1.18</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="9">
         <v>9999</v>
       </c>
       <c r="K10" s="2" t="s">
@@ -7166,26 +7233,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -7232,110 +7299,110 @@
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="L3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="M3" s="5" t="s">
+      <c r="L3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="M3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>30001</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>1</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>1</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>10</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -7345,16 +7412,16 @@
         <v>249</v>
       </c>
       <c r="I5" s="2"/>
-      <c r="J5" s="7">
+      <c r="J5" s="9">
         <v>5</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="9">
         <v>0.6</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="9">
         <v>10</v>
       </c>
-      <c r="M5" s="7">
+      <c r="M5" s="9">
         <v>1.35</v>
       </c>
       <c r="N5" s="2" t="s">
@@ -7362,22 +7429,22 @@
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>30002</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="9">
         <v>2</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <v>11</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <v>20</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -7387,16 +7454,16 @@
         <v>252</v>
       </c>
       <c r="I6" s="2"/>
-      <c r="J6" s="7">
+      <c r="J6" s="9">
         <v>11</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="9">
         <v>0.6</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="9">
         <v>201</v>
       </c>
-      <c r="M6" s="7">
+      <c r="M6" s="9">
         <v>1.35</v>
       </c>
       <c r="N6" s="2" t="s">
@@ -7404,22 +7471,22 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>30003</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="9">
         <v>3</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <v>21</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="9">
         <v>30</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -7429,16 +7496,16 @@
         <v>254</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="7">
+      <c r="J7" s="9">
         <v>17</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="9">
         <v>0.6</v>
       </c>
-      <c r="L7" s="7">
+      <c r="L7" s="9">
         <v>4042</v>
       </c>
-      <c r="M7" s="7">
+      <c r="M7" s="9">
         <v>1.35</v>
       </c>
       <c r="N7" s="2" t="s">
@@ -7446,22 +7513,22 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>30004</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="9">
         <v>4</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <v>31</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="9">
         <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
@@ -7471,16 +7538,16 @@
       <c r="I8" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <v>35</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="9">
         <v>1</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="9">
         <v>81285</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="9">
         <v>1.35</v>
       </c>
       <c r="N8" s="2" t="s">
@@ -7488,22 +7555,22 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>30005</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="9">
         <v>5</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <v>41</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="9">
         <v>50</v>
       </c>
       <c r="G9" s="2" t="s">
@@ -7513,16 +7580,16 @@
         <v>260</v>
       </c>
       <c r="I9" s="2"/>
-      <c r="J9" s="7">
+      <c r="J9" s="9">
         <v>29</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="9">
         <v>0.6</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="9">
         <v>1634371</v>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="9">
         <v>1.35</v>
       </c>
       <c r="N9" s="2" t="s">
@@ -7553,18 +7620,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -7593,62 +7660,62 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>31001</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -7657,13 +7724,13 @@
       <c r="D5" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>40007</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>15</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>667</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -7671,10 +7738,10 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>31002</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -7683,13 +7750,13 @@
       <c r="D6" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <v>40008</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="9">
         <v>33</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <v>148142</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -7721,22 +7788,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -7771,74 +7838,74 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>32001</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -7847,30 +7914,30 @@
       <c r="D5" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>40009</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>2</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="9">
         <v>15</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="9">
         <v>1.22</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="9">
         <v>9999</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="9">
         <v>2</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="9">
         <v>32002</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -7879,30 +7946,30 @@
       <c r="D6" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <v>40010</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <v>2</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="9">
         <v>15</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="9">
         <v>1.22</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="9">
         <v>9999</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="9">
         <v>3</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="9">
         <v>32003</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -7911,30 +7978,30 @@
       <c r="D7" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <v>40011</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <v>2</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="9">
         <v>15</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="9">
         <v>1.22</v>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="9">
         <v>9999</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="9">
         <v>4</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <v>32004</v>
       </c>
       <c r="C8" s="2" t="s">
@@ -7943,30 +8010,30 @@
       <c r="D8" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <v>40012</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <v>2</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="9">
         <v>15</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="9">
         <v>1.22</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="9">
         <v>9999</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="9">
         <v>5</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="9">
         <v>32005</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -7975,22 +8042,22 @@
       <c r="D9" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <v>40013</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="9">
         <v>2</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="9">
         <v>15</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="9">
         <v>1.22</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="9">
         <v>9999</v>
       </c>
     </row>
@@ -8019,17 +8086,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -8061,89 +8128,89 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="G3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>33001</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>1</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>40014</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>0.05</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>10</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="9">
         <v>1.25</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="9">
         <v>9999</v>
       </c>
     </row>
@@ -8173,16 +8240,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -8217,95 +8284,95 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="A3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="H3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="9">
         <v>34001</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <v>20</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <v>2</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="9">
         <v>7200</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>1.5</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="9">
         <v>10</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="9">
         <v>5</v>
       </c>
       <c r="J5" s="2" t="s">

</xml_diff>

<commit_message>
Add relic system UI with grade-sorted grid and detail popup
Builds the 무기고 > 유물 tab: slot status, gacha pull, and a
grade-sorted grid (matching the weapon grid) that opens a detail
popup for activate/deactivate, mirroring the weapon detail modal.
Wires active relic effects (stat bonus, gold gain %, time heist
cooldown reduction) into battle rewards, offline rewards, and time
heist, and confirms rebirth clears owned/active relics while slot
count (derived from exist tree progress) persists.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -46,7 +46,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'TimeHeistTable'!$A$4:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$Q$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'StringTable'!$A$4:$E$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'StringTable'!$A$4:$E$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7943,12 +7943,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="20.2" customWidth="1" min="3" max="3"/>
+    <col width="22.1" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
@@ -10088,8 +10088,238 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="6" t="n">
+        <v>40094</v>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>유물 뽑기</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Pull Relic</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="B95" s="6" t="n">
+        <v>40095</v>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>중복 환급</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate Refund</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n">
+        <v>92</v>
+      </c>
+      <c r="B96" s="6" t="n">
+        <v>40096</v>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>다음 슬롯</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Next Slot</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>40097</v>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>활성 슬롯</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Active Slots</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="B98" s="6" t="n">
+        <v>40098</v>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>보유 유물</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Owned Relics</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B99" s="6" t="n">
+        <v>40099</v>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>슬롯이 가득 참</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Slots Full</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="B100" s="6" t="n">
+        <v>40100</v>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>골드 획득량</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Gold Gain</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" s="6" t="n">
+        <v>40101</v>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>타임 하이스트 쿨타임</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Time Heist Cooldown</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>RelicUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" s="6" t="n">
+        <v>40102</v>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>활성화</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Activate</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" s="6" t="n">
+        <v>40103</v>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>비활성화</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Deactivate</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Button</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E93"/>
+  <autoFilter ref="A4:E103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Move weapon mastery UI to a growth-tab sub-tab, split by type
Adds a [스탯]/[숙련] sub-tab switcher to the growth panel and rebuilds
the mastery screen there: per-type (검/창/활) level, effect multiplier,
next-level cost, and an individual max button, with the currently
equipped weapon's type highlighted since only its mastery applies in
combat. maxUpgradeMastery now takes an optional weapon type so each
row can be maxed independently instead of only all-at-once.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -46,7 +46,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'TimeHeistTable'!$A$4:$J$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$Q$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'StringTable'!$A$4:$E$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'StringTable'!$A$4:$E$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7943,7 +7943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10318,8 +10318,54 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="6" t="n">
+        <v>40104</v>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>스탯</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Stat</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>GrowthUi</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" s="6" t="n">
+        <v>40105</v>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>숙련</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Mastery</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>GrowthUi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E103"/>
+  <autoFilter ref="A4:E105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Replace rebirth diamond formula with a stage-range reward table
The exponential DiamondBase/DiamondExponent formula is gone from
RebirthTable; diamond reward now comes from RebirthRewardTable, a
5-row table mapping stage ranges to fixed payouts. Lets the payout
curve be tuned directly in the spreadsheet instead of via a formula,
and the rebirth modal now previews the next tier's stage threshold
and payout so the reader can see rewards grow with depth.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -24,11 +24,12 @@
     <sheet name="RelicSlotTable" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="TimeHeistTable" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="RebirthTable" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="CommonTable" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="StringTable" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="RebirthRewardTable" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="CommonTable" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="StringTable" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'#TableDefine'!$A$1:$F$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'#TableDefine'!$A$1:$F$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'#EnumDefine'!$A$1:$D$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'StageTable'!$A$4:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'StatTable'!$A$4:$K$10</definedName>
@@ -44,9 +45,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'RelicTable'!$A$4:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'RelicSlotTable'!$A$4:$E$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'TimeHeistTable'!$A$4:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$R$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'StringTable'!$A$4:$E$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$P$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'RebirthRewardTable'!$A$4:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$125</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -529,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4584,12 +4586,12 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>다이아 지급 계수</t>
+          <t>포인트당 환급 증폭률</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>DiamondBase</t>
+          <t>RefundBonusPerPoint</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -4599,7 +4601,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>리버스 시 신규 지급되는 다이아 공식의 기준 계수. 지급량 = floor(DiamondBase × 도달스테이지^DiamondExponent). 환급이 아니라 신규 지급이라 rebirthSpent/환급 배율과 무관</t>
+          <t>누적 보너스 포인트 1당 리버스 환급량에 곱연산으로 붙는 증폭률(%). 환급 배율 = 1 + (누적 포인트 × 이 값 / 100). 전투 중 재화 획득량/스탯에는 영향 없음</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr"/>
@@ -4612,12 +4614,12 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>다이아 지급 지수</t>
+          <t>환급 배율 상한</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>DiamondExponent</t>
+          <t>MaxRefundMultiplier</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -4627,7 +4629,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>다이아 지급 공식에서 도달 스테이지에 적용하는 지수</t>
+          <t>환급 배율이 이 값을 넘지 않도록 제한</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr"/>
@@ -4640,22 +4642,22 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>포인트당 환급 증폭률</t>
+          <t>보너스 설명</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>RefundBonusPerPoint</t>
+          <t>//BonusDescription</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>누적 보너스 포인트 1당 리버스 환급량에 곱연산으로 붙는 증폭률(%). 환급 배율 = 1 + (누적 포인트 × 이 값 / 100). 전투 중 재화 획득량/스탯에는 영향 없음</t>
+          <t>회차 보너스 공식에 대한 참고 설명 (파싱 제외)</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr"/>
@@ -4663,27 +4665,27 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>RebirthTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>환급 배율 상한</t>
+          <t>순번</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>MaxRefundMultiplier</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>환급 배율이 이 값을 넘지 않도록 제한</t>
+          <t>행 순번(표시용)</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr"/>
@@ -4691,27 +4693,27 @@
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>RebirthTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>보너스 설명</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>//BonusDescription</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>회차 보너스 공식에 대한 참고 설명 (파싱 제외)</t>
+          <t>리버스 다이아 보상 구간 고유 ID (35100번대)</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr"/>
@@ -4719,27 +4721,27 @@
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>CommonTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>순번</t>
+          <t>이름</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>//Name</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>행 순번(표시용)</t>
+          <t>구간 설명 (파싱 제외)</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr"/>
@@ -4747,17 +4749,17 @@
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>CommonTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>구간 시작 스테이지</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>StageFrom</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -4767,7 +4769,7 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>공용 상수 고유 ID (36000번대)</t>
+          <t>이 구간의 시작 스테이지(포함)</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr"/>
@@ -4775,27 +4777,27 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>CommonTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>키</t>
+          <t>구간 끝 스테이지</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Key</t>
+          <t>StageTo</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>코드가 참조하는 식별자. 절대 수정 금지</t>
+          <t>이 구간의 끝 스테이지(포함). 마지막 구간은 999999로 열어둔다</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr"/>
@@ -4803,27 +4805,27 @@
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>CommonTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>이름</t>
+          <t>다이아 지급량</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>//Name</t>
+          <t>DiamondReward</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>행 구분용 참고 이름 (파싱 제외)</t>
+          <t>리버스 시점의 도달 스테이지가 이 구간에 속하면 지급되는 다이아 수량(고정값)</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr"/>
@@ -4831,27 +4833,27 @@
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>CommonTable</t>
+          <t>RebirthRewardTable</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>값</t>
+          <t>설명</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>//Description</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>실제 값. 수정 대상</t>
+          <t>행에 대한 참고 설명 (파싱 제외)</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr"/>
@@ -4864,22 +4866,22 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>값 타입</t>
+          <t>순번</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>ValueType</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Value를 int/float 중 무엇으로 해석할지</t>
+          <t>행 순번(표시용)</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr"/>
@@ -4892,22 +4894,22 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>설명</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>//Description</t>
+          <t>Id</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>행에 대한 참고 설명 (파싱 제외)</t>
+          <t>공용 상수 고유 ID (36000번대)</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr"/>
@@ -4915,27 +4917,27 @@
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>StringTable</t>
+          <t>CommonTable</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>순번</t>
+          <t>키</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Key</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>행 순번(표시용)</t>
+          <t>코드가 참조하는 식별자. 절대 수정 금지</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr"/>
@@ -4943,27 +4945,27 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>StringTable</t>
+          <t>CommonTable</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>이름</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t>//Name</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>문자열 고유 ID (40000번대). 다른 테이블의 이름ID가 참조</t>
+          <t>행 구분용 참고 이름 (파싱 제외)</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr"/>
@@ -4971,27 +4973,27 @@
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>StringTable</t>
+          <t>CommonTable</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>한국어</t>
+          <t>값</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>KOR</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>한국어 표시 문자열</t>
+          <t>실제 값. 수정 대상</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr"/>
@@ -4999,17 +5001,17 @@
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>StringTable</t>
+          <t>CommonTable</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>영문</t>
+          <t>값 타입</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>ValueType</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -5019,7 +5021,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>영문/내부 키 표시 문자열</t>
+          <t>Value를 int/float 중 무엇으로 해석할지</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr"/>
@@ -5027,17 +5029,17 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>StringTable</t>
+          <t>CommonTable</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>분류</t>
+          <t>설명</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>//Category</t>
+          <t>//Description</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -5047,7 +5049,7 @@
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>문자열 용도 분류 (파싱 제외)</t>
+          <t>행에 대한 참고 설명 (파싱 제외)</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr"/>
@@ -5055,23 +5057,27 @@
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>#EnumDefine</t>
+          <t>StringTable</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>enum 그룹</t>
-        </is>
-      </c>
-      <c r="C161" s="2" t="inlineStr"/>
+          <t>순번</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>enum 값이 속한 그룹 이름</t>
+          <t>행 순번(표시용)</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr"/>
@@ -5079,23 +5085,27 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>#EnumDefine</t>
+          <t>StringTable</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>한글 라벨</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr"/>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>기획 문서/화면에 쓰는 한글 표기</t>
+          <t>문자열 고유 ID (40000번대). 다른 테이블의 이름ID가 참조</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr"/>
@@ -5103,15 +5113,19 @@
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>#EnumDefine</t>
+          <t>StringTable</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>영문 라벨</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr"/>
+          <t>한국어</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>KOR</t>
+        </is>
+      </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
           <t>string</t>
@@ -5119,7 +5133,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>코드가 참조하는 영문 값</t>
+          <t>한국어 표시 문자열</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr"/>
@@ -5127,29 +5141,157 @@
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
+          <t>StringTable</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>영문</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>ENG</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>영문/내부 키 표시 문자열</t>
+        </is>
+      </c>
+      <c r="F164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>StringTable</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>분류</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>//Category</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>문자열 용도 분류 (파싱 제외)</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
           <t>#EnumDefine</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>enum 그룹</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr"/>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>enum 값이 속한 그룹 이름</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>#EnumDefine</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>한글 라벨</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr"/>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>기획 문서/화면에 쓰는 한글 표기</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>#EnumDefine</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>영문 라벨</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>코드가 참조하는 영문 값</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>#EnumDefine</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
         <is>
           <t>사용처</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr"/>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="C169" s="2" t="inlineStr"/>
+      <c r="D169" s="2" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="E164" s="2" t="inlineStr">
+      <c r="E169" s="2" t="inlineStr">
         <is>
           <t>이 enum 그룹을 참조하는 테이블.칼럼 목록</t>
         </is>
       </c>
-      <c r="F164" s="2" t="inlineStr"/>
+      <c r="F169" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F164"/>
+  <autoFilter ref="A1:F169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7113,7 +7255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7129,11 +7271,9 @@
     <col width="60" customWidth="1" min="11" max="11"/>
     <col width="18.3" customWidth="1" min="12" max="12"/>
     <col width="18.3" customWidth="1" min="13" max="13"/>
-    <col width="18.3" customWidth="1" min="14" max="14"/>
-    <col width="18.3" customWidth="1" min="15" max="15"/>
-    <col width="22.1" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="22.1" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7153,8 +7293,6 @@
       <c r="N1" s="3" t="n"/>
       <c r="O1" s="3" t="n"/>
       <c r="P1" s="3" t="n"/>
-      <c r="Q1" s="3" t="n"/>
-      <c r="R1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -7224,25 +7362,15 @@
       </c>
       <c r="N2" s="1" t="inlineStr">
         <is>
-          <t>다이아 지급 계수</t>
+          <t>포인트당 환급 증폭률</t>
         </is>
       </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>다이아 지급 지수</t>
+          <t>환급 배율 상한</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr">
-        <is>
-          <t>포인트당 환급 증폭률</t>
-        </is>
-      </c>
-      <c r="Q2" s="1" t="inlineStr">
-        <is>
-          <t>환급 배율 상한</t>
-        </is>
-      </c>
-      <c r="R2" s="1" t="inlineStr">
         <is>
           <t>보너스 설명</t>
         </is>
@@ -7326,16 +7454,6 @@
       </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="R3" s="4" t="inlineStr">
-        <is>
           <t>string</t>
         </is>
       </c>
@@ -7408,25 +7526,15 @@
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>DiamondBase</t>
+          <t>RefundBonusPerPoint</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
-          <t>DiamondExponent</t>
+          <t>MaxRefundMultiplier</t>
         </is>
       </c>
       <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>RefundBonusPerPoint</t>
-        </is>
-      </c>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>MaxRefundMultiplier</t>
-        </is>
-      </c>
-      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>//BonusDescription</t>
         </is>
@@ -7467,7 +7575,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>스테이지/스탯/숙련 초기화 + 소비 재화 전액 환급 + 다이아 신규 지급. 존재력 트리는 유지</t>
+          <t>스테이지/스탯/숙련 초기화 + 소비 재화 전액 환급 + 다이아 신규 지급(RebirthRewardTable). 존재력 트리는 유지</t>
         </is>
       </c>
       <c r="L5" s="6" t="n">
@@ -7477,30 +7585,283 @@
         <v>0.5</v>
       </c>
       <c r="N5" s="6" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>포인트 = 1.0 × 도달스테이지^0.5 (소수점 유지, 최소 스테이지 제한 없음). 다이아 지급량 = floor(20.0 × 도달스테이지^0.6, 환급과 무관한 신규 지급). 환급 배율 = 1 + (누적 포인트 × 1.0 / 100), 최대 5.0배. 전투 중 재화 획득량/스탯에는 영향 없음</t>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>포인트 = 1.0 × 도달스테이지^0.5 (소수점 유지, 최소 스테이지 제한 없음). 환급 배율 = 1 + (누적 포인트 × 1.0 / 100), 최대 5.0배. 전투 중 재화 획득량/스탯에는 영향 없음. 다이아 신규 지급량은 RebirthRewardTable(구간별 고정값)에서 조회한다</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:R5"/>
+  <autoFilter ref="A4:P5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="13.6" customWidth="1" min="3" max="3"/>
+    <col width="20.2" customWidth="1" min="4" max="4"/>
+    <col width="18.3" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="n"/>
+      <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>순번</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>구간 시작 스테이지</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>구간 끝 스테이지</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>다이아 지급량</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>설명</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Index</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>//Name</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>StageFrom</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>StageTo</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>DiamondReward</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>//Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>35101</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>1구간</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>35102</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2구간</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>35103</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>3구간</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>99</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>700</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>35104</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>4구간</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>199</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>35105</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>5구간(최종)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>999999</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7985,7 +8346,842 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20.1" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>enum 그룹</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>한글 라벨</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>영문 라벨</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>사용처</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CurrencyType</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>존재력</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>EXIST</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.GrantCurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>CurrencyType</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>성장에너지</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GROWTH_ENERGY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.GrantCurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>CurrencyType</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>숙련의정수</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>MASTERY_ESSENCE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.GrantCurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>CurrencyType</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>시간에너지</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>TIME_ENERGY</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.GrantCurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>CurrencyType</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>골드</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>GOLD</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.GrantCurrency</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>공격력</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>방어력</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>공격속도</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ASPD</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>치명타확률</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>CRIT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>치명타피해</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>CRIT_DMG</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>StatType</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>존재력획득량</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>EXIST_GAIN</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>NodeEffectType</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>스탯상승</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>STAT</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>NodeEffectType</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>재화지급</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>GRANT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ExistTreeTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>StageType</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>StageTable.StageType</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>StageType</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>보스</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Boss</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>StageTable.StageType</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>FeatureType</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>리버스</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>REBIRTH</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>FeatureUnlockTable.FeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FeatureType</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>타임하이스트</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>TIME_HEIST</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>FeatureUnlockTable.FeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>WeaponType</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>검</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Sword</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>WeaponTypeTable.WeaponType</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>WeaponType</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>창</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Spear</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>WeaponTypeTable.WeaponType</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>WeaponType</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>활</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Bow</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>WeaponTypeTable.WeaponType</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGrade</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>노말</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGradeTable.WeaponGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGrade</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>레어</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGradeTable.WeaponGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGrade</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>에픽</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGradeTable.WeaponGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGrade</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>유니크</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGradeTable.WeaponGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGrade</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>레전드리</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Legendary</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>WeaponGradeTable.WeaponGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>RelicGrade</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>노말</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.RelicGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>RelicGrade</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>레어</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.RelicGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>RelicGrade</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>에픽</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.RelicGrade</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>공격력</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>STAT_ATK</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>방어력</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>STAT_DEF</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>공격속도</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>STAT_ASPD</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>치명타확률</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>STAT_CRIT</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>치명타피해</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>STAT_CRIT_DMG</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>존재력획득량</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>STAT_EXIST_GAIN</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>골드획득량</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>GOLD_GAIN</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>RelicEffectType</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>타임하이스트쿨타임</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>TIMEHEIST_COOLDOWN</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>RelicTable.EffectType</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D37"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10874,841 +12070,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:E125"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20.1" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>enum 그룹</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>한글 라벨</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>영문 라벨</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>사용처</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>CurrencyType</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>존재력</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>EXIST</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.GrantCurrency</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>CurrencyType</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>성장에너지</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>GROWTH_ENERGY</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.GrantCurrency</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>CurrencyType</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>숙련의정수</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>MASTERY_ESSENCE</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.GrantCurrency</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>CurrencyType</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>시간에너지</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>TIME_ENERGY</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.GrantCurrency</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>CurrencyType</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>골드</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>GOLD</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.GrantCurrency</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>공격력</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>ATK</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>방어력</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>공격속도</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>ASPD</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>치명타확률</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>CRIT</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>치명타피해</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>CRIT_DMG</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>StatType</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>존재력획득량</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>EXIST_GAIN</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>NodeEffectType</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>스탯상승</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>STAT</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>NodeEffectType</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>재화지급</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>GRANT</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>ExistTreeTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>StageType</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>StageTable.StageType</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>StageType</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>보스</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Boss</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>StageTable.StageType</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>FeatureType</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>리버스</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>REBIRTH</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>FeatureUnlockTable.FeatureType</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>FeatureType</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>타임하이스트</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>TIME_HEIST</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>FeatureUnlockTable.FeatureType</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>WeaponType</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>검</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sword</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>WeaponTypeTable.WeaponType</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>WeaponType</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>창</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Spear</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>WeaponTypeTable.WeaponType</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>WeaponType</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>활</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Bow</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>WeaponTypeTable.WeaponType</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGrade</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>노말</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGrade</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>레어</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGrade</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>에픽</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGrade</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>유니크</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGrade</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>레전드리</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Legendary</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>RelicGrade</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>노말</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.RelicGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>RelicGrade</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>레어</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Rare</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.RelicGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>RelicGrade</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>에픽</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.RelicGrade</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>공격력</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>STAT_ATK</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>방어력</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>STAT_DEF</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>공격속도</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>STAT_ASPD</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>치명타확률</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>STAT_CRIT</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>치명타피해</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>STAT_CRIT_DMG</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>존재력획득량</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>STAT_EXIST_GAIN</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>골드획득량</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>GOLD_GAIN</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>타임하이스트쿨타임</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>TIMEHEIST_COOLDOWN</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rename Gacha to Summon and split it into weapon/relic sub-tabs
Renames the 가챠 tab to 소환 (StringTable rows 40028/40088) and gives
it the same [무기]/[유물] sub-tab structure the armory tab already
uses for [장비]/[유물] — pulling now lives entirely under Summon,
while the armory's relic tab keeps only slot management and the owned
grid. Moves weapon-gacha UI into systems/gacha/WeaponGachaTab.tsx and
extracts the relic-pull section that used to live inside RelicTab.tsx
into systems/gacha/RelicGachaTab.tsx, with SummonPanel.tsx as the new
container (replacing WeaponGachaPanel.tsx). Verified the new header
matches the armory's pixel-for-pixel and that pulls on both sub-tabs
correctly update state the armory tab reads back.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -48,7 +48,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'RebirthRewardTable'!$A$4:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$125</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9187,7 +9187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E125"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9777,12 +9777,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>가챠</t>
+          <t>소환</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Gacha</t>
+          <t>Summon</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -11157,12 +11157,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>가챠 레벨</t>
+          <t>소환 레벨</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Gacha Level</t>
+          <t>Summon Level</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -12068,8 +12068,31 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" s="6" t="n">
+        <v>122</v>
+      </c>
+      <c r="B126" s="6" t="n">
+        <v>40128</v>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>무기</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>GachaUi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E125"/>
+  <autoFilter ref="A4:E126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove dead DEF stat, restructure exist tree, fix rebirth multiplier timing
Fix three balance structure issues found by measurement: DEF had zero
gameplay effect since there's no player-damage-taken mechanic, so remove
it entirely (6->5 stats) and swap the one relic that used it (STAT_DEF ->
STAT_ASPD, renamed to match). Split each exist-tree tier from one row
into two sub-band rows so effects mix within a tier instead of ten
identical nodes in a row, reusing the existing range-matching lookup with
zero code changes; the new bands keep the exact same cost curve as
before and repeat ATK/ASPD to help the late-chapter pacing bottleneck
found earlier. Also make a rebirth's own reached-stage bonus apply to
that same rebirth's refund multiplier instead of only the next one, so
the first-ever rebirth isn't always stuck at x1.00 regardless of depth.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -30,10 +30,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'#TableDefine'!$A$1:$F$169</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'#EnumDefine'!$A$1:$D$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'#EnumDefine'!$A$1:$D$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'StageTable'!$A$4:$N$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'StatTable'!$A$4:$K$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ExistTreeTable'!$A$4:$N$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'StatTable'!$A$4:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ExistTreeTable'!$A$4:$N$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'FeatureUnlockTable'!$A$4:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'MasteryTable'!$A$4:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'WeaponTypeTable'!$A$4:$H$7</definedName>
@@ -48,7 +48,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'RebirthRewardTable'!$A$4:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6620,11 +6620,11 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>STAT_DEF</t>
+          <t>STAT_ASPD</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>40</v>
@@ -8352,7 +8352,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>방어력</t>
+          <t>공격속도</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ASPD</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -8545,12 +8545,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>공격속도</t>
+          <t>치명타확률</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>ASPD</t>
+          <t>CRIT</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -8567,12 +8567,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>치명타확률</t>
+          <t>치명타피해</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>CRIT</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -8589,12 +8589,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>치명타피해</t>
+          <t>존재력획득량</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>EXIST_GAIN</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -8606,22 +8606,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>StatType</t>
+          <t>NodeEffectType</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>존재력획득량</t>
+          <t>스탯상승</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>EXIST_GAIN</t>
+          <t>STAT</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>StatTable.StatType, ExistTreeTable.StatType, WeaponTypeTable.PrimaryStat</t>
+          <t>ExistTreeTable.EffectType</t>
         </is>
       </c>
     </row>
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>스탯상승</t>
+          <t>재화지급</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>STAT</t>
+          <t>GRANT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -8650,22 +8650,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NodeEffectType</t>
+          <t>StageType</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>재화지급</t>
+          <t>일반</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GRANT</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ExistTreeTable.EffectType</t>
+          <t>StageTable.StageType</t>
         </is>
       </c>
     </row>
@@ -8677,12 +8677,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>보스</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -8694,22 +8694,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>StageType</t>
+          <t>FeatureType</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>보스</t>
+          <t>리버스</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>REBIRTH</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>StageTable.StageType</t>
+          <t>FeatureUnlockTable.FeatureType</t>
         </is>
       </c>
     </row>
@@ -8721,12 +8721,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>리버스</t>
+          <t>타임하이스트</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>REBIRTH</t>
+          <t>TIME_HEIST</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -8738,22 +8738,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>FeatureType</t>
+          <t>WeaponType</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>타임하이스트</t>
+          <t>검</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>TIME_HEIST</t>
+          <t>Sword</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>FeatureUnlockTable.FeatureType</t>
+          <t>WeaponTypeTable.WeaponType</t>
         </is>
       </c>
     </row>
@@ -8765,12 +8765,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>검</t>
+          <t>창</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Sword</t>
+          <t>Spear</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -8787,12 +8787,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>창</t>
+          <t>활</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Spear</t>
+          <t>Bow</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -8804,22 +8804,22 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>WeaponType</t>
+          <t>WeaponGrade</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>활</t>
+          <t>노말</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>WeaponTypeTable.WeaponType</t>
+          <t>WeaponGradeTable.WeaponGrade</t>
         </is>
       </c>
     </row>
@@ -8831,12 +8831,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>노말</t>
+          <t>레어</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -8853,12 +8853,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>레어</t>
+          <t>에픽</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -8875,12 +8875,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>에픽</t>
+          <t>유니크</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Unique</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -8897,12 +8897,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>유니크</t>
+          <t>레전드리</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Legendary</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -8914,22 +8914,22 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>WeaponGrade</t>
+          <t>RelicGrade</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>레전드리</t>
+          <t>노말</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Legendary</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>WeaponGradeTable.WeaponGrade</t>
+          <t>RelicTable.RelicGrade</t>
         </is>
       </c>
     </row>
@@ -8941,12 +8941,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>노말</t>
+          <t>레어</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -8963,12 +8963,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>레어</t>
+          <t>에픽</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -8980,22 +8980,22 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>RelicGrade</t>
+          <t>RelicEffectType</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>에픽</t>
+          <t>공격력</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>STAT_ATK</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>RelicTable.RelicGrade</t>
+          <t>RelicTable.EffectType</t>
         </is>
       </c>
     </row>
@@ -9007,12 +9007,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>공격력</t>
+          <t>공격속도</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>STAT_ATK</t>
+          <t>STAT_ASPD</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -9029,12 +9029,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>방어력</t>
+          <t>치명타확률</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>STAT_DEF</t>
+          <t>STAT_CRIT</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -9051,12 +9051,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>공격속도</t>
+          <t>치명타피해</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>STAT_ASPD</t>
+          <t>STAT_CRIT_DMG</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -9073,12 +9073,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>치명타확률</t>
+          <t>존재력획득량</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>STAT_CRIT</t>
+          <t>STAT_EXIST_GAIN</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -9095,12 +9095,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>치명타피해</t>
+          <t>골드획득량</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>STAT_CRIT_DMG</t>
+          <t>GOLD_GAIN</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9117,12 +9117,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>존재력획득량</t>
+          <t>타임하이스트쿨타임</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>STAT_EXIST_GAIN</t>
+          <t>TIMEHEIST_COOLDOWN</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9131,52 +9131,8 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>골드획득량</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>GOLD_GAIN</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>RelicEffectType</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>타임하이스트쿨타임</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>TIMEHEIST_COOLDOWN</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>RelicTable.EffectType</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D37"/>
+  <autoFilter ref="A1:D35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9187,7 +9143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9313,16 +9269,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>40002</v>
+        <v>40003</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>방어력</t>
+          <t>공격속도</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ASPD</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -9336,16 +9292,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>40003</v>
+        <v>40004</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>공격속도</t>
+          <t>치명타 확률</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ASPD</t>
+          <t>CRIT</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -9359,16 +9315,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>40004</v>
+        <v>40005</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>치명타 확률</t>
+          <t>치명타피해</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>CRIT</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -9382,16 +9338,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>40005</v>
+        <v>40006</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>치명타피해</t>
+          <t>존재력 획득량</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>EXIST_GAIN</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -9405,21 +9361,21 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>40006</v>
+        <v>40007</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>존재력 획득량</t>
+          <t>리버스</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>EXIST_GAIN</t>
+          <t>REBIRTH</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Stat</t>
+          <t>System</t>
         </is>
       </c>
     </row>
@@ -9428,16 +9384,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>40007</v>
+        <v>40008</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>리버스</t>
+          <t>타임 하이스트</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>REBIRTH</t>
+          <t>TIME_HEIST</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -9451,21 +9407,21 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>40008</v>
+        <v>40015</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>타임 하이스트</t>
+          <t>존재력</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>TIME_HEIST</t>
+          <t>EXIST</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Currency</t>
         </is>
       </c>
     </row>
@@ -9474,16 +9430,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>40015</v>
+        <v>40016</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>존재력</t>
+          <t>성장에너지</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>EXIST</t>
+          <t>GROWTH_ENERGY</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -9497,16 +9453,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>40016</v>
+        <v>40017</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>성장에너지</t>
+          <t>숙련의 정수</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>GROWTH_ENERGY</t>
+          <t>MASTERY_ESSENCE</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -9520,16 +9476,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>40017</v>
+        <v>40018</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>숙련의 정수</t>
+          <t>시간에너지</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>MASTERY_ESSENCE</t>
+          <t>TIME_ENERGY</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -9543,16 +9499,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>40018</v>
+        <v>40019</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>시간에너지</t>
+          <t>골드</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>TIME_ENERGY</t>
+          <t>GOLD</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -9566,21 +9522,21 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>40019</v>
+        <v>40020</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>골드</t>
+          <t>존재력 트리</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>GOLD</t>
+          <t>EXIST_TREE</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>System</t>
         </is>
       </c>
     </row>
@@ -9589,21 +9545,21 @@
         <v>14</v>
       </c>
       <c r="B18" s="6" t="n">
-        <v>40020</v>
+        <v>40021</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>존재력 트리</t>
+          <t>존재</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>EXIST_TREE</t>
+          <t>EXIST_ABBR</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>CurrencyAbbr</t>
         </is>
       </c>
     </row>
@@ -9612,16 +9568,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>40021</v>
+        <v>40022</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>존재</t>
+          <t>성장</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>EXIST_ABBR</t>
+          <t>GROWTH_ABBR</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -9635,16 +9591,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="6" t="n">
-        <v>40022</v>
+        <v>40023</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>성장</t>
+          <t>시간</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>GROWTH_ABBR</t>
+          <t>TIME_ABBR</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -9658,16 +9614,16 @@
         <v>17</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>40023</v>
+        <v>40024</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>시간</t>
+          <t>골드</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>TIME_ABBR</t>
+          <t>GOLD_ABBR</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -9681,16 +9637,16 @@
         <v>18</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>40024</v>
+        <v>40025</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>골드</t>
+          <t>정수</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>GOLD_ABBR</t>
+          <t>ESSENCE_ABBR</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -9704,21 +9660,21 @@
         <v>19</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>40025</v>
+        <v>40026</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>정수</t>
+          <t>성장</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ESSENCE_ABBR</t>
+          <t>Growth</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>CurrencyAbbr</t>
+          <t>Tab</t>
         </is>
       </c>
     </row>
@@ -9727,16 +9683,16 @@
         <v>20</v>
       </c>
       <c r="B24" s="6" t="n">
-        <v>40026</v>
+        <v>40027</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>성장</t>
+          <t>무기고</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Growth</t>
+          <t>Armory</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -9750,16 +9706,16 @@
         <v>21</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>40027</v>
+        <v>40028</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>무기고</t>
+          <t>소환</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Armory</t>
+          <t>Summon</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -9773,16 +9729,16 @@
         <v>22</v>
       </c>
       <c r="B26" s="6" t="n">
-        <v>40028</v>
+        <v>40029</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>소환</t>
+          <t>존재력</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Summon</t>
+          <t>ExistTree</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -9796,16 +9752,16 @@
         <v>23</v>
       </c>
       <c r="B27" s="6" t="n">
-        <v>40029</v>
+        <v>40030</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>존재력</t>
+          <t>도감</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ExistTree</t>
+          <t>Dogam</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -9819,21 +9775,21 @@
         <v>24</v>
       </c>
       <c r="B28" s="6" t="n">
-        <v>40030</v>
+        <v>40031</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>도감</t>
+          <t>닫기</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Dogam</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Tab</t>
+          <t>Button</t>
         </is>
       </c>
     </row>
@@ -9842,16 +9798,16 @@
         <v>25</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>40031</v>
+        <v>40032</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>닫기</t>
+          <t>취소</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -9865,16 +9821,16 @@
         <v>26</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>40032</v>
+        <v>40033</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>취소</t>
+          <t>확인</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -9888,16 +9844,16 @@
         <v>27</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>40033</v>
+        <v>40034</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>확인</t>
+          <t>실행</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>Execute</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -9911,16 +9867,16 @@
         <v>28</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>40034</v>
+        <v>40035</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>실행</t>
+          <t>강탈</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Execute</t>
+          <t>Steal</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -9934,16 +9890,16 @@
         <v>29</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>40035</v>
+        <v>40036</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>강탈</t>
+          <t>받기</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Steal</t>
+          <t>Claim</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -9957,16 +9913,16 @@
         <v>30</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>40036</v>
+        <v>40037</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>받기</t>
+          <t>해금</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Claim</t>
+          <t>Unlock</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -9980,16 +9936,16 @@
         <v>31</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>40037</v>
+        <v>40038</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>해금</t>
+          <t>강화</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Unlock</t>
+          <t>Enhance</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -10003,16 +9959,16 @@
         <v>32</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>40038</v>
+        <v>40039</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>강화</t>
+          <t>수련</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Enhance</t>
+          <t>Train</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -10026,16 +9982,16 @@
         <v>33</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>40039</v>
+        <v>40040</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>수련</t>
+          <t>업그레이드</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Train</t>
+          <t>Upgrade</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -10049,16 +10005,16 @@
         <v>34</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>40040</v>
+        <v>40041</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>업그레이드</t>
+          <t>최대로</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Upgrade</t>
+          <t>MaxAll</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -10072,16 +10028,16 @@
         <v>35</v>
       </c>
       <c r="B39" s="6" t="n">
-        <v>40041</v>
+        <v>40042</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>최대로</t>
+          <t>뒤로</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>MaxAll</t>
+          <t>Back</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -10095,21 +10051,21 @@
         <v>36</v>
       </c>
       <c r="B40" s="6" t="n">
-        <v>40042</v>
+        <v>40043</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>뒤로</t>
+          <t>잠김</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Back</t>
+          <t>Locked</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>State</t>
         </is>
       </c>
     </row>
@@ -10118,16 +10074,16 @@
         <v>37</v>
       </c>
       <c r="B41" s="6" t="n">
-        <v>40043</v>
+        <v>40044</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>잠김</t>
+          <t>해금됨</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Unlocked</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -10141,16 +10097,16 @@
         <v>38</v>
       </c>
       <c r="B42" s="6" t="n">
-        <v>40044</v>
+        <v>40045</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>해금됨</t>
+          <t>사용 가능</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Unlocked</t>
+          <t>Available</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -10164,16 +10120,16 @@
         <v>39</v>
       </c>
       <c r="B43" s="6" t="n">
-        <v>40045</v>
+        <v>40046</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>사용 가능</t>
+          <t>티어</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Tier</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -10187,16 +10143,16 @@
         <v>40</v>
       </c>
       <c r="B44" s="6" t="n">
-        <v>40046</v>
+        <v>40047</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>티어</t>
+          <t>효과</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Effect</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -10210,16 +10166,16 @@
         <v>41</v>
       </c>
       <c r="B45" s="6" t="n">
-        <v>40047</v>
+        <v>40048</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>효과</t>
+          <t>비용</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Effect</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -10233,21 +10189,21 @@
         <v>42</v>
       </c>
       <c r="B46" s="6" t="n">
-        <v>40048</v>
+        <v>40049</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>비용</t>
+          <t>회차 보너스</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>RebirthBonus</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>RebirthBonus</t>
         </is>
       </c>
     </row>
@@ -10256,16 +10212,16 @@
         <v>43</v>
       </c>
       <c r="B47" s="6" t="n">
-        <v>40049</v>
+        <v>40050</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>회차 보너스</t>
+          <t>현재 회차</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>RebirthBonus</t>
+          <t>CurrentCycle</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -10279,16 +10235,16 @@
         <v>44</v>
       </c>
       <c r="B48" s="6" t="n">
-        <v>40050</v>
+        <v>40051</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>현재 회차</t>
+          <t>누적 포인트</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>CurrentCycle</t>
+          <t>TotalPoints</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -10302,16 +10258,16 @@
         <v>45</v>
       </c>
       <c r="B49" s="6" t="n">
-        <v>40051</v>
+        <v>40052</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>누적 포인트</t>
+          <t>획득 예정 포인트</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>TotalPoints</t>
+          <t>PendingPoints</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -10325,16 +10281,16 @@
         <v>46</v>
       </c>
       <c r="B50" s="6" t="n">
-        <v>40052</v>
+        <v>40053</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>획득 예정 포인트</t>
+          <t>환급 배율</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>PendingPoints</t>
+          <t>RefundMultiplier</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -10348,16 +10304,16 @@
         <v>47</v>
       </c>
       <c r="B51" s="6" t="n">
-        <v>40053</v>
+        <v>40054</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>환급 배율</t>
+          <t>최고 도달 스테이지</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>RefundMultiplier</t>
+          <t>MaxStageReached</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -10371,21 +10327,21 @@
         <v>48</v>
       </c>
       <c r="B52" s="6" t="n">
-        <v>40054</v>
+        <v>40055</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>최고 도달 스테이지</t>
+          <t>검</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>MaxStageReached</t>
+          <t>Sword</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>RebirthBonus</t>
+          <t>WeaponType</t>
         </is>
       </c>
     </row>
@@ -10394,16 +10350,16 @@
         <v>49</v>
       </c>
       <c r="B53" s="6" t="n">
-        <v>40055</v>
+        <v>40056</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>검</t>
+          <t>창</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Sword</t>
+          <t>Spear</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -10417,16 +10373,16 @@
         <v>50</v>
       </c>
       <c r="B54" s="6" t="n">
-        <v>40056</v>
+        <v>40057</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>창</t>
+          <t>활</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Spear</t>
+          <t>Bow</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -10440,21 +10396,21 @@
         <v>51</v>
       </c>
       <c r="B55" s="6" t="n">
-        <v>40057</v>
+        <v>40058</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>활</t>
+          <t>노말</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Bow</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>WeaponType</t>
+          <t>WeaponGrade</t>
         </is>
       </c>
     </row>
@@ -10463,16 +10419,16 @@
         <v>52</v>
       </c>
       <c r="B56" s="6" t="n">
-        <v>40058</v>
+        <v>40059</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>노말</t>
+          <t>레어</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -10486,16 +10442,16 @@
         <v>53</v>
       </c>
       <c r="B57" s="6" t="n">
-        <v>40059</v>
+        <v>40060</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>레어</t>
+          <t>에픽</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -10509,16 +10465,16 @@
         <v>54</v>
       </c>
       <c r="B58" s="6" t="n">
-        <v>40060</v>
+        <v>40061</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>에픽</t>
+          <t>유니크</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Unique</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -10532,16 +10488,16 @@
         <v>55</v>
       </c>
       <c r="B59" s="6" t="n">
-        <v>40061</v>
+        <v>40062</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>유니크</t>
+          <t>레전드리</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Unique</t>
+          <t>Legendary</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -10555,21 +10511,21 @@
         <v>56</v>
       </c>
       <c r="B60" s="6" t="n">
-        <v>40062</v>
+        <v>40063</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>레전드리</t>
+          <t>힘의 유물</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Legendary</t>
+          <t>Relic of Strength</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>WeaponGrade</t>
+          <t>RelicName</t>
         </is>
       </c>
     </row>
@@ -10578,16 +10534,16 @@
         <v>57</v>
       </c>
       <c r="B61" s="6" t="n">
-        <v>40063</v>
+        <v>40064</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>힘의 유물</t>
+          <t>신속의 유물</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Relic of Strength</t>
+          <t>Relic of Swiftness</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -10601,16 +10557,16 @@
         <v>58</v>
       </c>
       <c r="B62" s="6" t="n">
-        <v>40064</v>
+        <v>40065</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>방패의 유물</t>
+          <t>행운의 유물</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Relic of Shield</t>
+          <t>Relic of Luck</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -10624,16 +10580,16 @@
         <v>59</v>
       </c>
       <c r="B63" s="6" t="n">
-        <v>40065</v>
+        <v>40066</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>행운의 유물</t>
+          <t>가속의 유물</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Relic of Luck</t>
+          <t>Relic of Haste</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -10647,16 +10603,16 @@
         <v>60</v>
       </c>
       <c r="B64" s="6" t="n">
-        <v>40066</v>
+        <v>40067</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>가속의 유물</t>
+          <t>파괴의 유물</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Relic of Haste</t>
+          <t>Relic of Destruction</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -10670,16 +10626,16 @@
         <v>61</v>
       </c>
       <c r="B65" s="6" t="n">
-        <v>40067</v>
+        <v>40068</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>파괴의 유물</t>
+          <t>상인의 유물</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Relic of Destruction</t>
+          <t>Relic of Merchant</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -10693,16 +10649,16 @@
         <v>62</v>
       </c>
       <c r="B66" s="6" t="n">
-        <v>40068</v>
+        <v>40069</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>상인의 유물</t>
+          <t>균열의 유물</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Relic of Merchant</t>
+          <t>Relic of Rift</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -10716,16 +10672,16 @@
         <v>63</v>
       </c>
       <c r="B67" s="6" t="n">
-        <v>40069</v>
+        <v>40070</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>균열의 유물</t>
+          <t>시간의 유물</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Relic of Rift</t>
+          <t>Relic of Time</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -10739,16 +10695,16 @@
         <v>64</v>
       </c>
       <c r="B68" s="6" t="n">
-        <v>40070</v>
+        <v>40071</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>시간의 유물</t>
+          <t>전능의 유물</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Relic of Time</t>
+          <t>Relic of Omnipotence</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -10762,21 +10718,21 @@
         <v>65</v>
       </c>
       <c r="B69" s="6" t="n">
-        <v>40071</v>
+        <v>40072</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>전능의 유물</t>
+          <t>검 숙련</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Relic of Omnipotence</t>
+          <t>Sword Mastery</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>RelicName</t>
+          <t>Mastery</t>
         </is>
       </c>
     </row>
@@ -10785,16 +10741,16 @@
         <v>66</v>
       </c>
       <c r="B70" s="6" t="n">
-        <v>40072</v>
+        <v>40073</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>검 숙련</t>
+          <t>창 숙련</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Sword Mastery</t>
+          <t>Spear Mastery</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -10808,16 +10764,16 @@
         <v>67</v>
       </c>
       <c r="B71" s="6" t="n">
-        <v>40073</v>
+        <v>40074</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>창 숙련</t>
+          <t>활 숙련</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Spear Mastery</t>
+          <t>Bow Mastery</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -10831,21 +10787,21 @@
         <v>68</v>
       </c>
       <c r="B72" s="6" t="n">
-        <v>40074</v>
+        <v>40075</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>활 숙련</t>
+          <t>다이아</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Bow Mastery</t>
+          <t>DIAMOND</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Mastery</t>
+          <t>Currency</t>
         </is>
       </c>
     </row>
@@ -10854,7 +10810,7 @@
         <v>69</v>
       </c>
       <c r="B73" s="6" t="n">
-        <v>40075</v>
+        <v>40076</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
@@ -10863,12 +10819,12 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>DIAMOND</t>
+          <t>DIAMOND_ABBR</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>CurrencyAbbr</t>
         </is>
       </c>
     </row>
@@ -10877,21 +10833,21 @@
         <v>70</v>
       </c>
       <c r="B74" s="6" t="n">
-        <v>40076</v>
+        <v>40077</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>다이아</t>
+          <t>장착</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>DIAMOND_ABBR</t>
+          <t>Equip</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>CurrencyAbbr</t>
+          <t>Button</t>
         </is>
       </c>
     </row>
@@ -10900,16 +10856,16 @@
         <v>71</v>
       </c>
       <c r="B75" s="6" t="n">
-        <v>40077</v>
+        <v>40078</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>장착</t>
+          <t>돌파</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Equip</t>
+          <t>Breakthrough</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -10923,16 +10879,16 @@
         <v>72</v>
       </c>
       <c r="B76" s="6" t="n">
-        <v>40078</v>
+        <v>40079</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>돌파</t>
+          <t>합성</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Breakthrough</t>
+          <t>Fuse</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -10946,21 +10902,21 @@
         <v>73</v>
       </c>
       <c r="B77" s="6" t="n">
-        <v>40079</v>
+        <v>40080</v>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>합성</t>
+          <t>장비</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Fuse</t>
+          <t>Equipment</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>WeaponUi</t>
         </is>
       </c>
     </row>
@@ -10969,16 +10925,16 @@
         <v>74</v>
       </c>
       <c r="B78" s="6" t="n">
-        <v>40080</v>
+        <v>40081</v>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>장비</t>
+          <t>유물</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Relic</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -10992,16 +10948,16 @@
         <v>75</v>
       </c>
       <c r="B79" s="6" t="n">
-        <v>40081</v>
+        <v>40082</v>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>유물</t>
+          <t>보유 효과</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Relic</t>
+          <t>Own Bonus</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -11015,16 +10971,16 @@
         <v>76</v>
       </c>
       <c r="B80" s="6" t="n">
-        <v>40082</v>
+        <v>40083</v>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>보유 효과</t>
+          <t>장착 효과</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Own Bonus</t>
+          <t>Equip Bonus</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -11038,16 +10994,16 @@
         <v>77</v>
       </c>
       <c r="B81" s="6" t="n">
-        <v>40083</v>
+        <v>40084</v>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>장착 효과</t>
+          <t>장착 중</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Equip Bonus</t>
+          <t>Equipped</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -11061,16 +11017,16 @@
         <v>78</v>
       </c>
       <c r="B82" s="6" t="n">
-        <v>40084</v>
+        <v>40085</v>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>장착 중</t>
+          <t>장착된 무기 없음</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Equipped</t>
+          <t>No Weapon Equipped</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -11084,16 +11040,16 @@
         <v>79</v>
       </c>
       <c r="B83" s="6" t="n">
-        <v>40085</v>
+        <v>40086</v>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>장착된 무기 없음</t>
+          <t>보유 개수</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>No Weapon Equipped</t>
+          <t>Owned Count</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -11107,16 +11063,16 @@
         <v>80</v>
       </c>
       <c r="B84" s="6" t="n">
-        <v>40086</v>
+        <v>40087</v>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>보유 개수</t>
+          <t>등급</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Owned Count</t>
+          <t>Grade</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -11130,21 +11086,21 @@
         <v>81</v>
       </c>
       <c r="B85" s="6" t="n">
-        <v>40087</v>
+        <v>40088</v>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>등급</t>
+          <t>소환 레벨</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Grade</t>
+          <t>Summon Level</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>WeaponUi</t>
+          <t>GachaUi</t>
         </is>
       </c>
     </row>
@@ -11153,16 +11109,16 @@
         <v>82</v>
       </c>
       <c r="B86" s="6" t="n">
-        <v>40088</v>
+        <v>40089</v>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>소환 레벨</t>
+          <t>다음 레벨까지</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Summon Level</t>
+          <t>To Next Level</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -11176,16 +11132,16 @@
         <v>83</v>
       </c>
       <c r="B87" s="6" t="n">
-        <v>40089</v>
+        <v>40090</v>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>다음 레벨까지</t>
+          <t>1회 뽑기</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>To Next Level</t>
+          <t>Pull x1</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -11199,16 +11155,16 @@
         <v>84</v>
       </c>
       <c r="B88" s="6" t="n">
-        <v>40090</v>
+        <v>40091</v>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>1회 뽑기</t>
+          <t>10회 뽑기</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Pull x1</t>
+          <t>Pull x10</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -11222,16 +11178,16 @@
         <v>85</v>
       </c>
       <c r="B89" s="6" t="n">
-        <v>40091</v>
+        <v>40092</v>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>10회 뽑기</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Pull x10</t>
+          <t>New</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -11245,16 +11201,16 @@
         <v>86</v>
       </c>
       <c r="B90" s="6" t="n">
-        <v>40092</v>
+        <v>40093</v>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>중복</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Duplicate</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -11268,21 +11224,21 @@
         <v>87</v>
       </c>
       <c r="B91" s="6" t="n">
-        <v>40093</v>
+        <v>40094</v>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>중복</t>
+          <t>유물 뽑기</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Duplicate</t>
+          <t>Pull Relic</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>GachaUi</t>
+          <t>RelicUi</t>
         </is>
       </c>
     </row>
@@ -11291,16 +11247,16 @@
         <v>88</v>
       </c>
       <c r="B92" s="6" t="n">
-        <v>40094</v>
+        <v>40095</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>유물 뽑기</t>
+          <t>중복 환급</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Pull Relic</t>
+          <t>Duplicate Refund</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -11314,16 +11270,16 @@
         <v>89</v>
       </c>
       <c r="B93" s="6" t="n">
-        <v>40095</v>
+        <v>40096</v>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>중복 환급</t>
+          <t>다음 슬롯</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Duplicate Refund</t>
+          <t>Next Slot</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -11337,16 +11293,16 @@
         <v>90</v>
       </c>
       <c r="B94" s="6" t="n">
-        <v>40096</v>
+        <v>40097</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>다음 슬롯</t>
+          <t>활성 슬롯</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Next Slot</t>
+          <t>Active Slots</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -11360,16 +11316,16 @@
         <v>91</v>
       </c>
       <c r="B95" s="6" t="n">
-        <v>40097</v>
+        <v>40098</v>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>활성 슬롯</t>
+          <t>보유 유물</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Active Slots</t>
+          <t>Owned Relics</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -11383,16 +11339,16 @@
         <v>92</v>
       </c>
       <c r="B96" s="6" t="n">
-        <v>40098</v>
+        <v>40099</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>보유 유물</t>
+          <t>슬롯이 가득 참</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Owned Relics</t>
+          <t>Slots Full</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -11406,16 +11362,16 @@
         <v>93</v>
       </c>
       <c r="B97" s="6" t="n">
-        <v>40099</v>
+        <v>40100</v>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>슬롯이 가득 참</t>
+          <t>골드 획득량</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Slots Full</t>
+          <t>Gold Gain</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -11429,16 +11385,16 @@
         <v>94</v>
       </c>
       <c r="B98" s="6" t="n">
-        <v>40100</v>
+        <v>40101</v>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>골드 획득량</t>
+          <t>타임 하이스트 쿨타임</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Gold Gain</t>
+          <t>Time Heist Cooldown</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -11452,21 +11408,21 @@
         <v>95</v>
       </c>
       <c r="B99" s="6" t="n">
-        <v>40101</v>
+        <v>40102</v>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>타임 하이스트 쿨타임</t>
+          <t>활성화</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Time Heist Cooldown</t>
+          <t>Activate</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>RelicUi</t>
+          <t>Button</t>
         </is>
       </c>
     </row>
@@ -11475,16 +11431,16 @@
         <v>96</v>
       </c>
       <c r="B100" s="6" t="n">
-        <v>40102</v>
+        <v>40103</v>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>활성화</t>
+          <t>비활성화</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Activate</t>
+          <t>Deactivate</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -11498,21 +11454,21 @@
         <v>97</v>
       </c>
       <c r="B101" s="6" t="n">
-        <v>40103</v>
+        <v>40104</v>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>비활성화</t>
+          <t>스탯</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Deactivate</t>
+          <t>Stat</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Button</t>
+          <t>GrowthUi</t>
         </is>
       </c>
     </row>
@@ -11521,16 +11477,16 @@
         <v>98</v>
       </c>
       <c r="B102" s="6" t="n">
-        <v>40104</v>
+        <v>40105</v>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>스탯</t>
+          <t>숙련</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Stat</t>
+          <t>Mastery</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -11544,21 +11500,21 @@
         <v>99</v>
       </c>
       <c r="B103" s="6" t="n">
-        <v>40105</v>
+        <v>40106</v>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>숙련</t>
+          <t>적 HP</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Mastery</t>
+          <t>Enemy HP</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>GrowthUi</t>
+          <t>CommonUi</t>
         </is>
       </c>
     </row>
@@ -11567,16 +11523,16 @@
         <v>100</v>
       </c>
       <c r="B104" s="6" t="n">
-        <v>40106</v>
+        <v>40107</v>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>적 HP</t>
+          <t>적 공격력</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Enemy HP</t>
+          <t>Enemy ATK</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -11590,16 +11546,16 @@
         <v>101</v>
       </c>
       <c r="B105" s="6" t="n">
-        <v>40107</v>
+        <v>40108</v>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>적 공격력</t>
+          <t>처치 진행도</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Enemy ATK</t>
+          <t>Kill Progress</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -11613,16 +11569,16 @@
         <v>102</v>
       </c>
       <c r="B106" s="6" t="n">
-        <v>40108</v>
+        <v>40109</v>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>처치 진행도</t>
+          <t>스테이지 보상 (처치당)</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Kill Progress</t>
+          <t>Stage Reward (per kill)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -11636,16 +11592,16 @@
         <v>103</v>
       </c>
       <c r="B107" s="6" t="n">
-        <v>40109</v>
+        <v>40110</v>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>스테이지 보상 (처치당)</t>
+          <t>회차</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Stage Reward (per kill)</t>
+          <t>Cycle</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -11659,16 +11615,16 @@
         <v>104</v>
       </c>
       <c r="B108" s="6" t="n">
-        <v>40110</v>
+        <v>40111</v>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>회차</t>
+          <t>오프라인 보상</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Cycle</t>
+          <t>Offline Reward</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -11682,16 +11638,16 @@
         <v>105</v>
       </c>
       <c r="B109" s="6" t="n">
-        <v>40111</v>
+        <v>40112</v>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>오프라인 보상</t>
+          <t>비운 시간</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Offline Reward</t>
+          <t>Time Away</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
@@ -11705,16 +11661,16 @@
         <v>106</v>
       </c>
       <c r="B110" s="6" t="n">
-        <v>40112</v>
+        <v>40113</v>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>비운 시간</t>
+          <t>최대</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Time Away</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -11728,16 +11684,16 @@
         <v>107</v>
       </c>
       <c r="B111" s="6" t="n">
-        <v>40113</v>
+        <v>40114</v>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>최대</t>
+          <t>인정</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Max</t>
+          <t>Recognized</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -11751,16 +11707,16 @@
         <v>108</v>
       </c>
       <c r="B112" s="6" t="n">
-        <v>40114</v>
+        <v>40115</v>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>인정</t>
+          <t>획득 재화</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Recognized</t>
+          <t>Rewards Earned</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -11774,16 +11730,16 @@
         <v>109</v>
       </c>
       <c r="B113" s="6" t="n">
-        <v>40115</v>
+        <v>40116</v>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>획득 재화</t>
+          <t>1회 비용</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Rewards Earned</t>
+          <t>Cost per Pull</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
@@ -11797,16 +11753,16 @@
         <v>110</v>
       </c>
       <c r="B114" s="6" t="n">
-        <v>40116</v>
+        <v>40117</v>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>1회 비용</t>
+          <t>종</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Cost per Pull</t>
+          <t>Kinds</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -11820,16 +11776,16 @@
         <v>111</v>
       </c>
       <c r="B115" s="6" t="n">
-        <v>40117</v>
+        <v>40118</v>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>종</t>
+          <t>노드</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Kinds</t>
+          <t>Nodes</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -11843,16 +11799,16 @@
         <v>112</v>
       </c>
       <c r="B116" s="6" t="n">
-        <v>40118</v>
+        <v>40119</v>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>노드</t>
+          <t>대상 스테이지</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Nodes</t>
+          <t>Target Stage</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -11866,16 +11822,16 @@
         <v>113</v>
       </c>
       <c r="B117" s="6" t="n">
-        <v>40119</v>
+        <v>40120</v>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>대상 스테이지</t>
+          <t>클리어 환산</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Target Stage</t>
+          <t>Clears Converted</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -11889,16 +11845,16 @@
         <v>114</v>
       </c>
       <c r="B118" s="6" t="n">
-        <v>40120</v>
+        <v>40121</v>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>클리어 환산</t>
+          <t>획득 예정</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Clears Converted</t>
+          <t>Expected Gain</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
@@ -11912,16 +11868,16 @@
         <v>115</v>
       </c>
       <c r="B119" s="6" t="n">
-        <v>40121</v>
+        <v>40122</v>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>획득 예정</t>
+          <t>소모</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Expected Gain</t>
+          <t>Consume</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -11935,16 +11891,16 @@
         <v>116</v>
       </c>
       <c r="B120" s="6" t="n">
-        <v>40122</v>
+        <v>40123</v>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>소모</t>
+          <t>사용 횟수</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Consume</t>
+          <t>Use Count</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -11958,16 +11914,16 @@
         <v>117</v>
       </c>
       <c r="B121" s="6" t="n">
-        <v>40123</v>
+        <v>40124</v>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>사용 횟수</t>
+          <t>쿨타임</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Use Count</t>
+          <t>Cooldown</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -11981,16 +11937,16 @@
         <v>118</v>
       </c>
       <c r="B122" s="6" t="n">
-        <v>40124</v>
+        <v>40125</v>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>쿨타임</t>
+          <t>회</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Cooldown</t>
+          <t>Times</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -12004,16 +11960,16 @@
         <v>119</v>
       </c>
       <c r="B123" s="6" t="n">
-        <v>40125</v>
+        <v>40126</v>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>회</t>
+          <t>등급 확률</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Times</t>
+          <t>Grade Probability</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -12027,16 +11983,16 @@
         <v>120</v>
       </c>
       <c r="B124" s="6" t="n">
-        <v>40126</v>
+        <v>40127</v>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>등급 확률</t>
+          <t>보유</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Grade Probability</t>
+          <t>Owned</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -12050,21 +12006,21 @@
         <v>121</v>
       </c>
       <c r="B125" s="6" t="n">
-        <v>40127</v>
+        <v>40128</v>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>보유</t>
+          <t>무기</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Owned</t>
+          <t>Weapon</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>CommonUi</t>
+          <t>GachaUi</t>
         </is>
       </c>
     </row>
@@ -12073,21 +12029,21 @@
         <v>122</v>
       </c>
       <c r="B126" s="6" t="n">
-        <v>40128</v>
+        <v>40129</v>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>무기</t>
+          <t>건너뛰기</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Weapon</t>
+          <t>Skip</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>GachaUi</t>
+          <t>Onboarding</t>
         </is>
       </c>
     </row>
@@ -12096,16 +12052,16 @@
         <v>123</v>
       </c>
       <c r="B127" s="6" t="n">
-        <v>40129</v>
+        <v>40130</v>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>건너뛰기</t>
+          <t>다음</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Next</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -12119,16 +12075,16 @@
         <v>124</v>
       </c>
       <c r="B128" s="6" t="n">
-        <v>40130</v>
+        <v>40131</v>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>다음</t>
+          <t>시작하기</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -12142,21 +12098,21 @@
         <v>125</v>
       </c>
       <c r="B129" s="6" t="n">
-        <v>40131</v>
+        <v>40132</v>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>시작하기</t>
+          <t>다음 특별 해금까지</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Until Next Special Unlock</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>ExistUi</t>
         </is>
       </c>
     </row>
@@ -12165,49 +12121,26 @@
         <v>126</v>
       </c>
       <c r="B130" s="6" t="n">
-        <v>40132</v>
+        <v>40133</v>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>다음 특별 해금까지</t>
+          <t>새 소식</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Until Next Special Unlock</t>
+          <t>New</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>ExistUi</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="6" t="n">
-        <v>127</v>
-      </c>
-      <c r="B131" s="6" t="n">
-        <v>40133</v>
-      </c>
-      <c r="C131" s="2" t="inlineStr">
-        <is>
-          <t>새 소식</t>
-        </is>
-      </c>
-      <c r="D131" s="2" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="E131" s="2" t="inlineStr">
-        <is>
           <t>Badge</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E131"/>
+  <autoFilter ref="A4:E130"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13445,7 +13378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13703,22 +13636,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>방어력</t>
+          <t>공격속도</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>ASPD</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>40002</v>
+        <v>40003</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>1</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>8</v>
@@ -13731,7 +13664,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>방어력(DEF) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
+          <t>공격속도(ASPD) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
         </is>
       </c>
     </row>
@@ -13744,22 +13677,22 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>공격속도</t>
+          <t>치명타확률</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ASPD</t>
+          <t>CRIT</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>40003</v>
+        <v>40004</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.05</v>
+        <v>0.5</v>
       </c>
       <c r="H7" s="6" t="n">
         <v>8</v>
@@ -13772,7 +13705,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>공격속도(ASPD) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
+          <t>치명타확률(CRIT) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
         </is>
       </c>
     </row>
@@ -13785,22 +13718,22 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>치명타확률</t>
+          <t>치명타피해</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>CRIT</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>40004</v>
+        <v>40005</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="H8" s="6" t="n">
         <v>8</v>
@@ -13813,7 +13746,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>치명타확률(CRIT) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
+          <t>치명타피해(CRIT_DMG) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
         </is>
       </c>
     </row>
@@ -13826,22 +13759,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>치명타피해</t>
+          <t>존재력획득량</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>CRIT_DMG</t>
+          <t>EXIST_GAIN</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>40005</v>
+        <v>40006</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>2</v>
+        <v>0.02</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>8</v>
@@ -13854,53 +13787,12 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>치명타피해(CRIT_DMG) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>20006</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>존재력획득량</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>EXIST_GAIN</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>40006</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>9999</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
           <t>존재력획득량(EXIST_GAIN) 성장 스탯. 원본 공식과 동일한 기준값/증가치</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K10"/>
+  <autoFilter ref="A4:K9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13911,12 +13803,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="25.1" customWidth="1" min="3" max="3"/>
+    <col width="41.69999999999999" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -13927,7 +13819,7 @@
     <col width="15.4" customWidth="1" min="11" max="11"/>
     <col width="11.6" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="18.8" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14183,7 +14075,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1티어: 공격력</t>
+          <t>1티어-A: 공격력</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
@@ -14193,7 +14085,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -14220,7 +14112,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>order 1~10 구간. 원본 노드별 5종 순환 효과를 티어 단위 단일 효과로 단순화함 — 다음 단계 리팩터링 시 재검토 필요</t>
+          <t>order 1~7 구간</t>
         </is>
       </c>
     </row>
@@ -14233,17 +14125,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2티어: 방어력</t>
+          <t>1티어-B: 치명타 확률</t>
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -14252,25 +14144,25 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>CRIT</t>
         </is>
       </c>
       <c r="I6" s="2" t="n"/>
       <c r="J6" s="6" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>0.6</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>201</v>
+        <v>81</v>
       </c>
       <c r="M6" s="6" t="n">
         <v>1.35</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>order 11~20 구간. 원본 노드별 5종 순환 효과를 티어 단위 단일 효과로 단순화함 — 다음 단계 리팩터링 시 재검토 필요</t>
+          <t>order 8~10 구간</t>
         </is>
       </c>
     </row>
@@ -14283,17 +14175,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>3티어: 공격속도</t>
+          <t>2티어-A: 공격속도</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -14307,20 +14199,20 @@
       </c>
       <c r="I7" s="2" t="n"/>
       <c r="J7" s="6" t="n">
-        <v>17</v>
+        <v>0.8</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>4042</v>
+        <v>201</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>1.35</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>order 21~30 구간. 원본 노드별 5종 순환 효과를 티어 단위 단일 효과로 단순화함 — 다음 단계 리팩터링 시 재검토 필요</t>
+          <t>order 11~16 구간</t>
         </is>
       </c>
     </row>
@@ -14333,17 +14225,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>4티어: 숙련의 정수 지급</t>
+          <t>2티어-B: 시간에너지 지급</t>
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -14353,24 +14245,24 @@
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>MASTERY_ESSENCE</t>
+          <t>TIME_ENERGY</t>
         </is>
       </c>
       <c r="J8" s="6" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>81285</v>
+        <v>1217</v>
       </c>
       <c r="M8" s="6" t="n">
         <v>1.35</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>order 31~40 구간. 원본 노드별 5종 순환 효과를 티어 단위 단일 효과로 단순화함 — 다음 단계 리팩터링 시 재검토 필요</t>
+          <t>order 17~20 구간</t>
         </is>
       </c>
     </row>
@@ -14383,17 +14275,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>5티어: 존재력획득량</t>
+          <t>3티어-A: 치명타피해</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -14402,30 +14294,280 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>EXIST_GAIN</t>
+          <t>CRIT_DMG</t>
         </is>
       </c>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="6" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>1634371</v>
+        <v>4042</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>1.35</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>order 41~50 구간. 원본 노드별 5종 순환 효과를 티어 단위 단일 효과로 단순화함 — 다음 단계 리팩터링 시 재검토 필요</t>
+          <t>order 21~26 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>30006</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>3티어-B: 숙련의 정수 지급</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>GRANT</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>MASTERY_ESSENCE</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>24472</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>order 27~30 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>30007</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>4티어-A: 공격력 (1티어-A 연장)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>STAT</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>ATK</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>81285</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>order 31~37 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>30008</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>4티어-B: 숙련의 정수 지급 (3티어-B 연장)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>GRANT</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>MASTERY_ESSENCE</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>664277</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>order 38~40 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>30009</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>5티어-A: 존재력획득량</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>STAT</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>EXIST_GAIN</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>1634371</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>order 41~46 구간</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>30010</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>5티어-B: 공격속도 (2티어-A 연장)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>STAT</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>ASPD</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>9893577</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>order 47~50 구간</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N9"/>
+  <autoFilter ref="A4:N14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Slow down exist tree checkpoint pacing and add growth auto-upgrade toggle
Node 15/rebirth was reachable in 3m34s and node 33/time heist in 5m50s,
well under the 5-7min / 11-15min targets. Raised the exist-tree node
cost curve (base 8->12, growth rate 1.16->1.13) and lowered exist_reward
(/2 -> /4.5) together so later nodes slow down proportionally more than
early ones, landing node15 at ~5m16s and node33/time-heist unlock at
~12-14min without regressing back to the previous multi-day pace.

Also added an auto-upgrade toggle to the growth tab so a live demo
doesn't require manually clicking every stat upgrade as growth energy
comes in. It always buys the cheapest of the 5 stats first and never
touches the exist tree, which stays a fully manual, player-driven loop
by design.
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -48,7 +48,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'RebirthTable'!$A$4:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'RebirthRewardTable'!$A$4:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'CommonTable'!$A$4:$G$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'StringTable'!$A$4:$E$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9143,7 +9143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -12139,8 +12139,31 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="6" t="n">
+        <v>127</v>
+      </c>
+      <c r="B131" s="6" t="n">
+        <v>40134</v>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>자동 업그레이드</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Auto Upgrade</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>GrowthUi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E130"/>
+  <autoFilter ref="A4:E131"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12490,7 +12513,7 @@
         <v>9</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L6" s="6" t="n">
         <v>15</v>
@@ -12538,7 +12561,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L7" s="6" t="n">
         <v>0</v>
@@ -12586,7 +12609,7 @@
         <v>24</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="L8" s="6" t="n">
         <v>20</v>
@@ -12634,7 +12657,7 @@
         <v>9</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>0</v>
@@ -12682,7 +12705,7 @@
         <v>54</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="L10" s="6" t="n">
         <v>25</v>
@@ -12730,7 +12753,7 @@
         <v>20</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="L11" s="6" t="n">
         <v>0</v>
@@ -12778,7 +12801,7 @@
         <v>120</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="L12" s="6" t="n">
         <v>30</v>
@@ -12826,7 +12849,7 @@
         <v>43</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="L13" s="6" t="n">
         <v>0</v>
@@ -12874,7 +12897,7 @@
         <v>258</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="L14" s="6" t="n">
         <v>35</v>
@@ -12922,7 +12945,7 @@
         <v>93</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="L15" s="6" t="n">
         <v>0</v>
@@ -12970,7 +12993,7 @@
         <v>561</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="L16" s="6" t="n">
         <v>40</v>
@@ -13018,7 +13041,7 @@
         <v>202</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="L17" s="6" t="n">
         <v>0</v>
@@ -13066,7 +13089,7 @@
         <v>1212</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="L18" s="6" t="n">
         <v>45</v>
@@ -13114,7 +13137,7 @@
         <v>437</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="L19" s="6" t="n">
         <v>0</v>
@@ -13162,7 +13185,7 @@
         <v>2619</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="L20" s="6" t="n">
         <v>50</v>
@@ -13210,7 +13233,7 @@
         <v>943</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="L21" s="6" t="n">
         <v>0</v>
@@ -13258,7 +13281,7 @@
         <v>5658</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="L22" s="6" t="n">
         <v>55</v>
@@ -13306,7 +13329,7 @@
         <v>2037</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="L23" s="6" t="n">
         <v>0</v>
@@ -13354,7 +13377,7 @@
         <v>12219</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="L24" s="6" t="n">
         <v>60</v>
@@ -14105,10 +14128,10 @@
         <v>0.6</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M5" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -14155,10 +14178,10 @@
         <v>0.6</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -14205,10 +14228,10 @@
         <v>0.15</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -14255,10 +14278,10 @@
         <v>2</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -14305,10 +14328,10 @@
         <v>1</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -14355,10 +14378,10 @@
         <v>1</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>379</v>
+        <v>287</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -14405,10 +14428,10 @@
         <v>0.6</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>686</v>
+        <v>469</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -14455,10 +14478,10 @@
         <v>1</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>1941</v>
+        <v>1104</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -14505,10 +14528,10 @@
         <v>0.6</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>3029</v>
+        <v>1593</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
@@ -14555,10 +14578,10 @@
         <v>0.15</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>7381</v>
+        <v>3317</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -14759,7 +14782,7 @@
         <v>15</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -14791,7 +14814,7 @@
         <v>33</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>924</v>
+        <v>599</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Lower weapon gacha pull cost to 30 diamond (v0.4.0)
Went 40 -> 60 (to offset the ~9.1x diamond supply increase) -> 50 (frozen
per request) -> 30 (asked to be more generous). Flat across all 8 gacha
levels, same as before.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -16414,7 +16414,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -16464,7 +16464,7 @@
         <v>3</v>
       </c>
       <c r="P6" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -16514,7 +16514,7 @@
         <v>5</v>
       </c>
       <c r="P7" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -16564,7 +16564,7 @@
         <v>8</v>
       </c>
       <c r="P8" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -16614,7 +16614,7 @@
         <v>12</v>
       </c>
       <c r="P9" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -16664,7 +16664,7 @@
         <v>16</v>
       </c>
       <c r="P10" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -16714,7 +16714,7 @@
         <v>22</v>
       </c>
       <c r="P11" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -16764,7 +16764,7 @@
         <v>30</v>
       </c>
       <c r="P12" s="8">
-        <v>60</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -53055,7 +53055,7 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E1" t="s">
         <v>1190</v>
       </c>

</xml_diff>

<commit_message>
Revert weapon gacha pull cost to 50 diamond (v0.4.0)
Lowering it to 30 last commit misread the request — the intent was to keep
players actually spending 50 diamond per pull, not cut it further.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -16414,7 +16414,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -16464,7 +16464,7 @@
         <v>3</v>
       </c>
       <c r="P6" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -16514,7 +16514,7 @@
         <v>5</v>
       </c>
       <c r="P7" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -16564,7 +16564,7 @@
         <v>8</v>
       </c>
       <c r="P8" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -16614,7 +16614,7 @@
         <v>12</v>
       </c>
       <c r="P9" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -16664,7 +16664,7 @@
         <v>16</v>
       </c>
       <c r="P10" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -16714,7 +16714,7 @@
         <v>22</v>
       </c>
       <c r="P11" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -16764,7 +16764,7 @@
         <v>30</v>
       </c>
       <c r="P12" s="8">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebalance Mythic gacha odds and scale down diamond supply (v0.4.0)
- Mythic weapon gacha weight now scales 0.03% (level 0) -> 0.100% (level 7,
  max) instead of climbing to ~4.7%. There's no grade above Mythic yet, so
  it should stay rare until one exists; the difference moves to Legendary.
  Every level's weight total is normalized to exactly 100 so each level's
  Mythic weight equals its percentage directly.
- Diamond supply (StageTable.FirstClearDiamond / RebirthRewardTable.
  DiamondReward) scaled back from ~9.1x to 4x the pre-v0.4.0 baseline
  (commit 5433c49) -- the earlier bump was too generous. Recomputed fresh
  from that commit's values each time rather than compounding multipliers,
  so rounding doesn't drift. Pull cost stays at 50.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -16489,7 +16489,7 @@
         <v>1.8</v>
       </c>
       <c r="I5" s="8">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="J5" s="8">
         <v>0.03</v>
@@ -16539,10 +16539,10 @@
         <v>3.3</v>
       </c>
       <c r="I6" s="8">
-        <v>0.7</v>
+        <v>0.66</v>
       </c>
       <c r="J6" s="8">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="K6" s="8">
         <v>50</v>
@@ -16589,10 +16589,10 @@
         <v>5.5</v>
       </c>
       <c r="I7" s="8">
-        <v>1.5</v>
+        <v>1.45</v>
       </c>
       <c r="J7" s="8">
-        <v>0.4</v>
+        <v>0.05</v>
       </c>
       <c r="K7" s="8">
         <v>42</v>
@@ -16639,10 +16639,10 @@
         <v>8</v>
       </c>
       <c r="I8" s="8">
-        <v>2</v>
+        <v>1.94</v>
       </c>
       <c r="J8" s="8">
-        <v>0.6</v>
+        <v>0.06</v>
       </c>
       <c r="K8" s="8">
         <v>35</v>
@@ -16689,10 +16689,10 @@
         <v>12</v>
       </c>
       <c r="I9" s="8">
-        <v>4</v>
+        <v>3.93</v>
       </c>
       <c r="J9" s="8">
-        <v>1.4</v>
+        <v>0.07</v>
       </c>
       <c r="K9" s="8">
         <v>28</v>
@@ -16739,10 +16739,10 @@
         <v>15</v>
       </c>
       <c r="I10" s="8">
-        <v>6</v>
+        <v>6.92</v>
       </c>
       <c r="J10" s="8">
-        <v>2.2</v>
+        <v>0.08</v>
       </c>
       <c r="K10" s="8">
         <v>23</v>
@@ -16789,10 +16789,10 @@
         <v>18</v>
       </c>
       <c r="I11" s="8">
-        <v>9</v>
+        <v>10.91</v>
       </c>
       <c r="J11" s="8">
-        <v>3.3</v>
+        <v>0.09</v>
       </c>
       <c r="K11" s="8">
         <v>19</v>
@@ -16839,10 +16839,10 @@
         <v>21</v>
       </c>
       <c r="I12" s="8">
-        <v>13</v>
+        <v>15.9</v>
       </c>
       <c r="J12" s="8">
-        <v>4.8</v>
+        <v>0.1</v>
       </c>
       <c r="K12" s="8">
         <v>15</v>
@@ -30677,7 +30677,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -30721,7 +30721,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -30765,7 +30765,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -30809,7 +30809,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -30853,7 +30853,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -30897,7 +30897,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -30941,7 +30941,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -30985,7 +30985,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -31029,7 +31029,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="8">
-        <v>56</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -31073,7 +31073,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="8">
-        <v>161</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -31117,7 +31117,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -31161,7 +31161,7 @@
         <v>0</v>
       </c>
       <c r="N16" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -31205,7 +31205,7 @@
         <v>0</v>
       </c>
       <c r="N17" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -31249,7 +31249,7 @@
         <v>0</v>
       </c>
       <c r="N18" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -31293,7 +31293,7 @@
         <v>0</v>
       </c>
       <c r="N19" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -31337,7 +31337,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -31381,7 +31381,7 @@
         <v>0</v>
       </c>
       <c r="N21" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -31425,7 +31425,7 @@
         <v>0</v>
       </c>
       <c r="N22" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -31469,7 +31469,7 @@
         <v>0</v>
       </c>
       <c r="N23" s="8">
-        <v>63</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -31513,7 +31513,7 @@
         <v>0</v>
       </c>
       <c r="N24" s="8">
-        <v>189</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -31557,7 +31557,7 @@
         <v>0</v>
       </c>
       <c r="N25" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -31601,7 +31601,7 @@
         <v>0</v>
       </c>
       <c r="N26" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -31645,7 +31645,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -31689,7 +31689,7 @@
         <v>0</v>
       </c>
       <c r="N28" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -31733,7 +31733,7 @@
         <v>0</v>
       </c>
       <c r="N29" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -31777,7 +31777,7 @@
         <v>0</v>
       </c>
       <c r="N30" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -31821,7 +31821,7 @@
         <v>0</v>
       </c>
       <c r="N31" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -31865,7 +31865,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -31909,7 +31909,7 @@
         <v>0</v>
       </c>
       <c r="N33" s="8">
-        <v>70</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -31953,7 +31953,7 @@
         <v>0</v>
       </c>
       <c r="N34" s="8">
-        <v>217</v>
+        <v>96</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -31997,7 +31997,7 @@
         <v>0</v>
       </c>
       <c r="N35" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -32041,7 +32041,7 @@
         <v>0</v>
       </c>
       <c r="N36" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -32085,7 +32085,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -32129,7 +32129,7 @@
         <v>0</v>
       </c>
       <c r="N38" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -32173,7 +32173,7 @@
         <v>0</v>
       </c>
       <c r="N39" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -32217,7 +32217,7 @@
         <v>0</v>
       </c>
       <c r="N40" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -32261,7 +32261,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -32305,7 +32305,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -32349,7 +32349,7 @@
         <v>0</v>
       </c>
       <c r="N43" s="8">
-        <v>91</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -32393,7 +32393,7 @@
         <v>0</v>
       </c>
       <c r="N44" s="8">
-        <v>273</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -32437,7 +32437,7 @@
         <v>0</v>
       </c>
       <c r="N45" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -32481,7 +32481,7 @@
         <v>0</v>
       </c>
       <c r="N46" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -32525,7 +32525,7 @@
         <v>0</v>
       </c>
       <c r="N47" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -32569,7 +32569,7 @@
         <v>0</v>
       </c>
       <c r="N48" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -32613,7 +32613,7 @@
         <v>0</v>
       </c>
       <c r="N49" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -32657,7 +32657,7 @@
         <v>0</v>
       </c>
       <c r="N50" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -32701,7 +32701,7 @@
         <v>0</v>
       </c>
       <c r="N51" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -32745,7 +32745,7 @@
         <v>0</v>
       </c>
       <c r="N52" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -32789,7 +32789,7 @@
         <v>0</v>
       </c>
       <c r="N53" s="8">
-        <v>112</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -32833,7 +32833,7 @@
         <v>0</v>
       </c>
       <c r="N54" s="8">
-        <v>329</v>
+        <v>144</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -32877,7 +32877,7 @@
         <v>0</v>
       </c>
       <c r="N55" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
@@ -32921,7 +32921,7 @@
         <v>0</v>
       </c>
       <c r="N56" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -32965,7 +32965,7 @@
         <v>0</v>
       </c>
       <c r="N57" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -33009,7 +33009,7 @@
         <v>0</v>
       </c>
       <c r="N58" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
@@ -33053,7 +33053,7 @@
         <v>0</v>
       </c>
       <c r="N59" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
@@ -33097,7 +33097,7 @@
         <v>0</v>
       </c>
       <c r="N60" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
@@ -33141,7 +33141,7 @@
         <v>0</v>
       </c>
       <c r="N61" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
@@ -33185,7 +33185,7 @@
         <v>0</v>
       </c>
       <c r="N62" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
@@ -33229,7 +33229,7 @@
         <v>0</v>
       </c>
       <c r="N63" s="8">
-        <v>126</v>
+        <v>56</v>
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
@@ -33273,7 +33273,7 @@
         <v>0</v>
       </c>
       <c r="N64" s="8">
-        <v>385</v>
+        <v>168</v>
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
@@ -33317,7 +33317,7 @@
         <v>0</v>
       </c>
       <c r="N65" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
@@ -33361,7 +33361,7 @@
         <v>0</v>
       </c>
       <c r="N66" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -33405,7 +33405,7 @@
         <v>0</v>
       </c>
       <c r="N67" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
@@ -33449,7 +33449,7 @@
         <v>0</v>
       </c>
       <c r="N68" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
@@ -33493,7 +33493,7 @@
         <v>0</v>
       </c>
       <c r="N69" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -33537,7 +33537,7 @@
         <v>0</v>
       </c>
       <c r="N70" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
@@ -33581,7 +33581,7 @@
         <v>0</v>
       </c>
       <c r="N71" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
@@ -33625,7 +33625,7 @@
         <v>0</v>
       </c>
       <c r="N72" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
@@ -33669,7 +33669,7 @@
         <v>0</v>
       </c>
       <c r="N73" s="8">
-        <v>147</v>
+        <v>64</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
@@ -33713,7 +33713,7 @@
         <v>0</v>
       </c>
       <c r="N74" s="8">
-        <v>434</v>
+        <v>192</v>
       </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
@@ -33757,7 +33757,7 @@
         <v>0</v>
       </c>
       <c r="N75" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
@@ -33801,7 +33801,7 @@
         <v>0</v>
       </c>
       <c r="N76" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.25">
@@ -33845,7 +33845,7 @@
         <v>0</v>
       </c>
       <c r="N77" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
@@ -33889,7 +33889,7 @@
         <v>0</v>
       </c>
       <c r="N78" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
@@ -33933,7 +33933,7 @@
         <v>0</v>
       </c>
       <c r="N79" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
@@ -33977,7 +33977,7 @@
         <v>0</v>
       </c>
       <c r="N80" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
@@ -34021,7 +34021,7 @@
         <v>0</v>
       </c>
       <c r="N81" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
@@ -34065,7 +34065,7 @@
         <v>0</v>
       </c>
       <c r="N82" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.25">
@@ -34109,7 +34109,7 @@
         <v>0</v>
       </c>
       <c r="N83" s="8">
-        <v>175</v>
+        <v>76</v>
       </c>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
@@ -34153,7 +34153,7 @@
         <v>0</v>
       </c>
       <c r="N84" s="8">
-        <v>518</v>
+        <v>228</v>
       </c>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
@@ -34197,7 +34197,7 @@
         <v>0</v>
       </c>
       <c r="N85" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
@@ -34241,7 +34241,7 @@
         <v>0</v>
       </c>
       <c r="N86" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
@@ -34285,7 +34285,7 @@
         <v>0</v>
       </c>
       <c r="N87" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
@@ -34329,7 +34329,7 @@
         <v>0</v>
       </c>
       <c r="N88" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
@@ -34373,7 +34373,7 @@
         <v>0</v>
       </c>
       <c r="N89" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -34417,7 +34417,7 @@
         <v>0</v>
       </c>
       <c r="N90" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -34461,7 +34461,7 @@
         <v>0</v>
       </c>
       <c r="N91" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
@@ -34505,7 +34505,7 @@
         <v>0</v>
       </c>
       <c r="N92" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
@@ -34549,7 +34549,7 @@
         <v>0</v>
       </c>
       <c r="N93" s="8">
-        <v>210</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
@@ -34593,7 +34593,7 @@
         <v>0</v>
       </c>
       <c r="N94" s="8">
-        <v>630</v>
+        <v>276</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
@@ -34637,7 +34637,7 @@
         <v>0</v>
       </c>
       <c r="N95" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -34681,7 +34681,7 @@
         <v>0</v>
       </c>
       <c r="N96" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
@@ -34725,7 +34725,7 @@
         <v>0</v>
       </c>
       <c r="N97" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
@@ -34769,7 +34769,7 @@
         <v>0</v>
       </c>
       <c r="N98" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
@@ -34813,7 +34813,7 @@
         <v>0</v>
       </c>
       <c r="N99" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
@@ -34857,7 +34857,7 @@
         <v>0</v>
       </c>
       <c r="N100" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
@@ -34901,7 +34901,7 @@
         <v>0</v>
       </c>
       <c r="N101" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
@@ -34945,7 +34945,7 @@
         <v>0</v>
       </c>
       <c r="N102" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.25">
@@ -34989,7 +34989,7 @@
         <v>0</v>
       </c>
       <c r="N103" s="8">
-        <v>245</v>
+        <v>108</v>
       </c>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.25">
@@ -35033,7 +35033,7 @@
         <v>0</v>
       </c>
       <c r="N104" s="8">
-        <v>735</v>
+        <v>324</v>
       </c>
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.25">
@@ -35077,7 +35077,7 @@
         <v>0</v>
       </c>
       <c r="N105" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.25">
@@ -35121,7 +35121,7 @@
         <v>0</v>
       </c>
       <c r="N106" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="107" spans="1:14" x14ac:dyDescent="0.25">
@@ -35165,7 +35165,7 @@
         <v>0</v>
       </c>
       <c r="N107" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.25">
@@ -35209,7 +35209,7 @@
         <v>0</v>
       </c>
       <c r="N108" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
@@ -35253,7 +35253,7 @@
         <v>0</v>
       </c>
       <c r="N109" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.25">
@@ -35297,7 +35297,7 @@
         <v>0</v>
       </c>
       <c r="N110" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.25">
@@ -35341,7 +35341,7 @@
         <v>0</v>
       </c>
       <c r="N111" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.25">
@@ -35385,7 +35385,7 @@
         <v>0</v>
       </c>
       <c r="N112" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.25">
@@ -35429,7 +35429,7 @@
         <v>0</v>
       </c>
       <c r="N113" s="8">
-        <v>280</v>
+        <v>124</v>
       </c>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.25">
@@ -35473,7 +35473,7 @@
         <v>0</v>
       </c>
       <c r="N114" s="8">
-        <v>847</v>
+        <v>372</v>
       </c>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.25">
@@ -35517,7 +35517,7 @@
         <v>0</v>
       </c>
       <c r="N115" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
@@ -35561,7 +35561,7 @@
         <v>0</v>
       </c>
       <c r="N116" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.25">
@@ -35605,7 +35605,7 @@
         <v>0</v>
       </c>
       <c r="N117" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.25">
@@ -35649,7 +35649,7 @@
         <v>0</v>
       </c>
       <c r="N118" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.25">
@@ -35693,7 +35693,7 @@
         <v>0</v>
       </c>
       <c r="N119" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.25">
@@ -35737,7 +35737,7 @@
         <v>0</v>
       </c>
       <c r="N120" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.25">
@@ -35781,7 +35781,7 @@
         <v>0</v>
       </c>
       <c r="N121" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.25">
@@ -35825,7 +35825,7 @@
         <v>0</v>
       </c>
       <c r="N122" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.25">
@@ -35869,7 +35869,7 @@
         <v>0</v>
       </c>
       <c r="N123" s="8">
-        <v>336</v>
+        <v>148</v>
       </c>
     </row>
     <row r="124" spans="1:14" x14ac:dyDescent="0.25">
@@ -35913,7 +35913,7 @@
         <v>0</v>
       </c>
       <c r="N124" s="8">
-        <v>1008</v>
+        <v>444</v>
       </c>
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.25">
@@ -35957,7 +35957,7 @@
         <v>0</v>
       </c>
       <c r="N125" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="126" spans="1:14" x14ac:dyDescent="0.25">
@@ -36001,7 +36001,7 @@
         <v>0</v>
       </c>
       <c r="N126" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.25">
@@ -36045,7 +36045,7 @@
         <v>0</v>
       </c>
       <c r="N127" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.25">
@@ -36089,7 +36089,7 @@
         <v>0</v>
       </c>
       <c r="N128" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.25">
@@ -36133,7 +36133,7 @@
         <v>0</v>
       </c>
       <c r="N129" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="130" spans="1:14" x14ac:dyDescent="0.25">
@@ -36177,7 +36177,7 @@
         <v>0</v>
       </c>
       <c r="N130" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.25">
@@ -36221,7 +36221,7 @@
         <v>0</v>
       </c>
       <c r="N131" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.25">
@@ -36265,7 +36265,7 @@
         <v>0</v>
       </c>
       <c r="N132" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="133" spans="1:14" x14ac:dyDescent="0.25">
@@ -36309,7 +36309,7 @@
         <v>0</v>
       </c>
       <c r="N133" s="8">
-        <v>399</v>
+        <v>176</v>
       </c>
     </row>
     <row r="134" spans="1:14" x14ac:dyDescent="0.25">
@@ -36353,7 +36353,7 @@
         <v>0</v>
       </c>
       <c r="N134" s="8">
-        <v>1204</v>
+        <v>528</v>
       </c>
     </row>
     <row r="135" spans="1:14" x14ac:dyDescent="0.25">
@@ -36397,7 +36397,7 @@
         <v>0</v>
       </c>
       <c r="N135" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="136" spans="1:14" x14ac:dyDescent="0.25">
@@ -36441,7 +36441,7 @@
         <v>0</v>
       </c>
       <c r="N136" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="137" spans="1:14" x14ac:dyDescent="0.25">
@@ -36485,7 +36485,7 @@
         <v>0</v>
       </c>
       <c r="N137" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="138" spans="1:14" x14ac:dyDescent="0.25">
@@ -36529,7 +36529,7 @@
         <v>0</v>
       </c>
       <c r="N138" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="139" spans="1:14" x14ac:dyDescent="0.25">
@@ -36573,7 +36573,7 @@
         <v>0</v>
       </c>
       <c r="N139" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="140" spans="1:14" x14ac:dyDescent="0.25">
@@ -36617,7 +36617,7 @@
         <v>0</v>
       </c>
       <c r="N140" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.25">
@@ -36661,7 +36661,7 @@
         <v>0</v>
       </c>
       <c r="N141" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.25">
@@ -36705,7 +36705,7 @@
         <v>0</v>
       </c>
       <c r="N142" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.25">
@@ -36749,7 +36749,7 @@
         <v>0</v>
       </c>
       <c r="N143" s="8">
-        <v>476</v>
+        <v>208</v>
       </c>
     </row>
     <row r="144" spans="1:14" x14ac:dyDescent="0.25">
@@ -36793,7 +36793,7 @@
         <v>0</v>
       </c>
       <c r="N144" s="8">
-        <v>1421</v>
+        <v>624</v>
       </c>
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.25">
@@ -36837,7 +36837,7 @@
         <v>0</v>
       </c>
       <c r="N145" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.25">
@@ -36881,7 +36881,7 @@
         <v>0</v>
       </c>
       <c r="N146" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.25">
@@ -36925,7 +36925,7 @@
         <v>0</v>
       </c>
       <c r="N147" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.25">
@@ -36969,7 +36969,7 @@
         <v>0</v>
       </c>
       <c r="N148" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="149" spans="1:14" x14ac:dyDescent="0.25">
@@ -37013,7 +37013,7 @@
         <v>0</v>
       </c>
       <c r="N149" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="150" spans="1:14" x14ac:dyDescent="0.25">
@@ -37057,7 +37057,7 @@
         <v>0</v>
       </c>
       <c r="N150" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="151" spans="1:14" x14ac:dyDescent="0.25">
@@ -37101,7 +37101,7 @@
         <v>0</v>
       </c>
       <c r="N151" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.25">
@@ -37145,7 +37145,7 @@
         <v>0</v>
       </c>
       <c r="N152" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.25">
@@ -37189,7 +37189,7 @@
         <v>0</v>
       </c>
       <c r="N153" s="8">
-        <v>553</v>
+        <v>244</v>
       </c>
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.25">
@@ -37233,7 +37233,7 @@
         <v>0</v>
       </c>
       <c r="N154" s="8">
-        <v>1666</v>
+        <v>732</v>
       </c>
     </row>
     <row r="155" spans="1:14" x14ac:dyDescent="0.25">
@@ -37277,7 +37277,7 @@
         <v>0</v>
       </c>
       <c r="N155" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="156" spans="1:14" x14ac:dyDescent="0.25">
@@ -37321,7 +37321,7 @@
         <v>0</v>
       </c>
       <c r="N156" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="157" spans="1:14" x14ac:dyDescent="0.25">
@@ -37365,7 +37365,7 @@
         <v>0</v>
       </c>
       <c r="N157" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="158" spans="1:14" x14ac:dyDescent="0.25">
@@ -37409,7 +37409,7 @@
         <v>0</v>
       </c>
       <c r="N158" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.25">
@@ -37453,7 +37453,7 @@
         <v>0</v>
       </c>
       <c r="N159" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="160" spans="1:14" x14ac:dyDescent="0.25">
@@ -37497,7 +37497,7 @@
         <v>0</v>
       </c>
       <c r="N160" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.25">
@@ -37541,7 +37541,7 @@
         <v>0</v>
       </c>
       <c r="N161" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.25">
@@ -37585,7 +37585,7 @@
         <v>0</v>
       </c>
       <c r="N162" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.25">
@@ -37629,7 +37629,7 @@
         <v>0</v>
       </c>
       <c r="N163" s="8">
-        <v>658</v>
+        <v>288</v>
       </c>
     </row>
     <row r="164" spans="1:14" x14ac:dyDescent="0.25">
@@ -37673,7 +37673,7 @@
         <v>0</v>
       </c>
       <c r="N164" s="8">
-        <v>1967</v>
+        <v>864</v>
       </c>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
@@ -37717,7 +37717,7 @@
         <v>0</v>
       </c>
       <c r="N165" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.25">
@@ -37761,7 +37761,7 @@
         <v>0</v>
       </c>
       <c r="N166" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.25">
@@ -37805,7 +37805,7 @@
         <v>0</v>
       </c>
       <c r="N167" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.25">
@@ -37849,7 +37849,7 @@
         <v>0</v>
       </c>
       <c r="N168" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.25">
@@ -37893,7 +37893,7 @@
         <v>0</v>
       </c>
       <c r="N169" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.25">
@@ -37937,7 +37937,7 @@
         <v>0</v>
       </c>
       <c r="N170" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.25">
@@ -37981,7 +37981,7 @@
         <v>0</v>
       </c>
       <c r="N171" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.25">
@@ -38025,7 +38025,7 @@
         <v>0</v>
       </c>
       <c r="N172" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="173" spans="1:14" x14ac:dyDescent="0.25">
@@ -38069,7 +38069,7 @@
         <v>0</v>
       </c>
       <c r="N173" s="8">
-        <v>777</v>
+        <v>340</v>
       </c>
     </row>
     <row r="174" spans="1:14" x14ac:dyDescent="0.25">
@@ -38113,7 +38113,7 @@
         <v>0</v>
       </c>
       <c r="N174" s="8">
-        <v>2324</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="175" spans="1:14" x14ac:dyDescent="0.25">
@@ -38157,7 +38157,7 @@
         <v>0</v>
       </c>
       <c r="N175" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="176" spans="1:14" x14ac:dyDescent="0.25">
@@ -38201,7 +38201,7 @@
         <v>0</v>
       </c>
       <c r="N176" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="177" spans="1:14" x14ac:dyDescent="0.25">
@@ -38245,7 +38245,7 @@
         <v>0</v>
       </c>
       <c r="N177" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="178" spans="1:14" x14ac:dyDescent="0.25">
@@ -38289,7 +38289,7 @@
         <v>0</v>
       </c>
       <c r="N178" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.25">
@@ -38333,7 +38333,7 @@
         <v>0</v>
       </c>
       <c r="N179" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.25">
@@ -38377,7 +38377,7 @@
         <v>0</v>
       </c>
       <c r="N180" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.25">
@@ -38421,7 +38421,7 @@
         <v>0</v>
       </c>
       <c r="N181" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="182" spans="1:14" x14ac:dyDescent="0.25">
@@ -38465,7 +38465,7 @@
         <v>0</v>
       </c>
       <c r="N182" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="183" spans="1:14" x14ac:dyDescent="0.25">
@@ -38509,7 +38509,7 @@
         <v>0</v>
       </c>
       <c r="N183" s="8">
-        <v>910</v>
+        <v>400</v>
       </c>
     </row>
     <row r="184" spans="1:14" x14ac:dyDescent="0.25">
@@ -38553,7 +38553,7 @@
         <v>0</v>
       </c>
       <c r="N184" s="8">
-        <v>2730</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="185" spans="1:14" x14ac:dyDescent="0.25">
@@ -38597,7 +38597,7 @@
         <v>0</v>
       </c>
       <c r="N185" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="186" spans="1:14" x14ac:dyDescent="0.25">
@@ -38641,7 +38641,7 @@
         <v>0</v>
       </c>
       <c r="N186" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="187" spans="1:14" x14ac:dyDescent="0.25">
@@ -38685,7 +38685,7 @@
         <v>0</v>
       </c>
       <c r="N187" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="188" spans="1:14" x14ac:dyDescent="0.25">
@@ -38729,7 +38729,7 @@
         <v>0</v>
       </c>
       <c r="N188" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="189" spans="1:14" x14ac:dyDescent="0.25">
@@ -38773,7 +38773,7 @@
         <v>0</v>
       </c>
       <c r="N189" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="190" spans="1:14" x14ac:dyDescent="0.25">
@@ -38817,7 +38817,7 @@
         <v>0</v>
       </c>
       <c r="N190" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="191" spans="1:14" x14ac:dyDescent="0.25">
@@ -38861,7 +38861,7 @@
         <v>0</v>
       </c>
       <c r="N191" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
@@ -38905,7 +38905,7 @@
         <v>0</v>
       </c>
       <c r="N192" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
@@ -38949,7 +38949,7 @@
         <v>0</v>
       </c>
       <c r="N193" s="8">
-        <v>1071</v>
+        <v>472</v>
       </c>
     </row>
     <row r="194" spans="1:14" x14ac:dyDescent="0.25">
@@ -38993,7 +38993,7 @@
         <v>0</v>
       </c>
       <c r="N194" s="8">
-        <v>3220</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="195" spans="1:14" x14ac:dyDescent="0.25">
@@ -39037,7 +39037,7 @@
         <v>0</v>
       </c>
       <c r="N195" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
@@ -39081,7 +39081,7 @@
         <v>0</v>
       </c>
       <c r="N196" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="197" spans="1:14" x14ac:dyDescent="0.25">
@@ -39125,7 +39125,7 @@
         <v>0</v>
       </c>
       <c r="N197" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.25">
@@ -39169,7 +39169,7 @@
         <v>0</v>
       </c>
       <c r="N198" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="199" spans="1:14" x14ac:dyDescent="0.25">
@@ -39213,7 +39213,7 @@
         <v>0</v>
       </c>
       <c r="N199" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="200" spans="1:14" x14ac:dyDescent="0.25">
@@ -39257,7 +39257,7 @@
         <v>0</v>
       </c>
       <c r="N200" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="201" spans="1:14" x14ac:dyDescent="0.25">
@@ -39301,7 +39301,7 @@
         <v>0</v>
       </c>
       <c r="N201" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="202" spans="1:14" x14ac:dyDescent="0.25">
@@ -39345,7 +39345,7 @@
         <v>0</v>
       </c>
       <c r="N202" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="203" spans="1:14" x14ac:dyDescent="0.25">
@@ -39389,7 +39389,7 @@
         <v>0</v>
       </c>
       <c r="N203" s="8">
-        <v>1267</v>
+        <v>556</v>
       </c>
     </row>
     <row r="204" spans="1:14" x14ac:dyDescent="0.25">
@@ -39433,7 +39433,7 @@
         <v>0</v>
       </c>
       <c r="N204" s="8">
-        <v>3794</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="205" spans="1:14" x14ac:dyDescent="0.25">
@@ -39477,7 +39477,7 @@
         <v>0</v>
       </c>
       <c r="N205" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="206" spans="1:14" x14ac:dyDescent="0.25">
@@ -39521,7 +39521,7 @@
         <v>0</v>
       </c>
       <c r="N206" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
@@ -39565,7 +39565,7 @@
         <v>0</v>
       </c>
       <c r="N207" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
@@ -39609,7 +39609,7 @@
         <v>0</v>
       </c>
       <c r="N208" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.25">
@@ -39653,7 +39653,7 @@
         <v>0</v>
       </c>
       <c r="N209" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="210" spans="1:14" x14ac:dyDescent="0.25">
@@ -39697,7 +39697,7 @@
         <v>0</v>
       </c>
       <c r="N210" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.25">
@@ -39741,7 +39741,7 @@
         <v>0</v>
       </c>
       <c r="N211" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="212" spans="1:14" x14ac:dyDescent="0.25">
@@ -39785,7 +39785,7 @@
         <v>0</v>
       </c>
       <c r="N212" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="213" spans="1:14" x14ac:dyDescent="0.25">
@@ -39829,7 +39829,7 @@
         <v>0</v>
       </c>
       <c r="N213" s="8">
-        <v>1491</v>
+        <v>656</v>
       </c>
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.25">
@@ -39873,7 +39873,7 @@
         <v>0</v>
       </c>
       <c r="N214" s="8">
-        <v>4480</v>
+        <v>1968</v>
       </c>
     </row>
     <row r="215" spans="1:14" x14ac:dyDescent="0.25">
@@ -39917,7 +39917,7 @@
         <v>0</v>
       </c>
       <c r="N215" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="216" spans="1:14" x14ac:dyDescent="0.25">
@@ -39961,7 +39961,7 @@
         <v>0</v>
       </c>
       <c r="N216" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="217" spans="1:14" x14ac:dyDescent="0.25">
@@ -40005,7 +40005,7 @@
         <v>0</v>
       </c>
       <c r="N217" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="218" spans="1:14" x14ac:dyDescent="0.25">
@@ -40049,7 +40049,7 @@
         <v>0</v>
       </c>
       <c r="N218" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="219" spans="1:14" x14ac:dyDescent="0.25">
@@ -40093,7 +40093,7 @@
         <v>0</v>
       </c>
       <c r="N219" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="220" spans="1:14" x14ac:dyDescent="0.25">
@@ -40137,7 +40137,7 @@
         <v>0</v>
       </c>
       <c r="N220" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="221" spans="1:14" x14ac:dyDescent="0.25">
@@ -40181,7 +40181,7 @@
         <v>0</v>
       </c>
       <c r="N221" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="222" spans="1:14" x14ac:dyDescent="0.25">
@@ -40225,7 +40225,7 @@
         <v>0</v>
       </c>
       <c r="N222" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="223" spans="1:14" x14ac:dyDescent="0.25">
@@ -40269,7 +40269,7 @@
         <v>0</v>
       </c>
       <c r="N223" s="8">
-        <v>1764</v>
+        <v>776</v>
       </c>
     </row>
     <row r="224" spans="1:14" x14ac:dyDescent="0.25">
@@ -40313,7 +40313,7 @@
         <v>0</v>
       </c>
       <c r="N224" s="8">
-        <v>5299</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="225" spans="1:14" x14ac:dyDescent="0.25">
@@ -40357,7 +40357,7 @@
         <v>0</v>
       </c>
       <c r="N225" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="226" spans="1:14" x14ac:dyDescent="0.25">
@@ -40401,7 +40401,7 @@
         <v>0</v>
       </c>
       <c r="N226" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="227" spans="1:14" x14ac:dyDescent="0.25">
@@ -40445,7 +40445,7 @@
         <v>0</v>
       </c>
       <c r="N227" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="228" spans="1:14" x14ac:dyDescent="0.25">
@@ -40489,7 +40489,7 @@
         <v>0</v>
       </c>
       <c r="N228" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="229" spans="1:14" x14ac:dyDescent="0.25">
@@ -40533,7 +40533,7 @@
         <v>0</v>
       </c>
       <c r="N229" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="230" spans="1:14" x14ac:dyDescent="0.25">
@@ -40577,7 +40577,7 @@
         <v>0</v>
       </c>
       <c r="N230" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="231" spans="1:14" x14ac:dyDescent="0.25">
@@ -40621,7 +40621,7 @@
         <v>0</v>
       </c>
       <c r="N231" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="232" spans="1:14" x14ac:dyDescent="0.25">
@@ -40665,7 +40665,7 @@
         <v>0</v>
       </c>
       <c r="N232" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="233" spans="1:14" x14ac:dyDescent="0.25">
@@ -40709,7 +40709,7 @@
         <v>0</v>
       </c>
       <c r="N233" s="8">
-        <v>2086</v>
+        <v>916</v>
       </c>
     </row>
     <row r="234" spans="1:14" x14ac:dyDescent="0.25">
@@ -40753,7 +40753,7 @@
         <v>0</v>
       </c>
       <c r="N234" s="8">
-        <v>6251</v>
+        <v>2748</v>
       </c>
     </row>
     <row r="235" spans="1:14" x14ac:dyDescent="0.25">
@@ -40797,7 +40797,7 @@
         <v>0</v>
       </c>
       <c r="N235" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="236" spans="1:14" x14ac:dyDescent="0.25">
@@ -40841,7 +40841,7 @@
         <v>0</v>
       </c>
       <c r="N236" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="237" spans="1:14" x14ac:dyDescent="0.25">
@@ -40885,7 +40885,7 @@
         <v>0</v>
       </c>
       <c r="N237" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="238" spans="1:14" x14ac:dyDescent="0.25">
@@ -40929,7 +40929,7 @@
         <v>0</v>
       </c>
       <c r="N238" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="239" spans="1:14" x14ac:dyDescent="0.25">
@@ -40973,7 +40973,7 @@
         <v>0</v>
       </c>
       <c r="N239" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="240" spans="1:14" x14ac:dyDescent="0.25">
@@ -41017,7 +41017,7 @@
         <v>0</v>
       </c>
       <c r="N240" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="241" spans="1:14" x14ac:dyDescent="0.25">
@@ -41061,7 +41061,7 @@
         <v>0</v>
       </c>
       <c r="N241" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="242" spans="1:14" x14ac:dyDescent="0.25">
@@ -41105,7 +41105,7 @@
         <v>0</v>
       </c>
       <c r="N242" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="243" spans="1:14" x14ac:dyDescent="0.25">
@@ -41149,7 +41149,7 @@
         <v>0</v>
       </c>
       <c r="N243" s="8">
-        <v>2457</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="244" spans="1:14" x14ac:dyDescent="0.25">
@@ -41193,7 +41193,7 @@
         <v>0</v>
       </c>
       <c r="N244" s="8">
-        <v>7371</v>
+        <v>3240</v>
       </c>
     </row>
     <row r="245" spans="1:14" x14ac:dyDescent="0.25">
@@ -41237,7 +41237,7 @@
         <v>0</v>
       </c>
       <c r="N245" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="246" spans="1:14" x14ac:dyDescent="0.25">
@@ -41281,7 +41281,7 @@
         <v>0</v>
       </c>
       <c r="N246" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="247" spans="1:14" x14ac:dyDescent="0.25">
@@ -41325,7 +41325,7 @@
         <v>0</v>
       </c>
       <c r="N247" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="248" spans="1:14" x14ac:dyDescent="0.25">
@@ -41369,7 +41369,7 @@
         <v>0</v>
       </c>
       <c r="N248" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="249" spans="1:14" x14ac:dyDescent="0.25">
@@ -41413,7 +41413,7 @@
         <v>0</v>
       </c>
       <c r="N249" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="250" spans="1:14" x14ac:dyDescent="0.25">
@@ -41457,7 +41457,7 @@
         <v>0</v>
       </c>
       <c r="N250" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="251" spans="1:14" x14ac:dyDescent="0.25">
@@ -41501,7 +41501,7 @@
         <v>0</v>
       </c>
       <c r="N251" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="252" spans="1:14" x14ac:dyDescent="0.25">
@@ -41545,7 +41545,7 @@
         <v>0</v>
       </c>
       <c r="N252" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="253" spans="1:14" x14ac:dyDescent="0.25">
@@ -41589,7 +41589,7 @@
         <v>0</v>
       </c>
       <c r="N253" s="8">
-        <v>2905</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="254" spans="1:14" x14ac:dyDescent="0.25">
@@ -41633,7 +41633,7 @@
         <v>0</v>
       </c>
       <c r="N254" s="8">
-        <v>8708</v>
+        <v>3828</v>
       </c>
     </row>
     <row r="255" spans="1:14" x14ac:dyDescent="0.25">
@@ -41677,7 +41677,7 @@
         <v>0</v>
       </c>
       <c r="N255" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="256" spans="1:14" x14ac:dyDescent="0.25">
@@ -41721,7 +41721,7 @@
         <v>0</v>
       </c>
       <c r="N256" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="257" spans="1:14" x14ac:dyDescent="0.25">
@@ -41765,7 +41765,7 @@
         <v>0</v>
       </c>
       <c r="N257" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="258" spans="1:14" x14ac:dyDescent="0.25">
@@ -41809,7 +41809,7 @@
         <v>0</v>
       </c>
       <c r="N258" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="259" spans="1:14" x14ac:dyDescent="0.25">
@@ -41853,7 +41853,7 @@
         <v>0</v>
       </c>
       <c r="N259" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="260" spans="1:14" x14ac:dyDescent="0.25">
@@ -41897,7 +41897,7 @@
         <v>0</v>
       </c>
       <c r="N260" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="261" spans="1:14" x14ac:dyDescent="0.25">
@@ -41941,7 +41941,7 @@
         <v>0</v>
       </c>
       <c r="N261" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="262" spans="1:14" x14ac:dyDescent="0.25">
@@ -41985,7 +41985,7 @@
         <v>0</v>
       </c>
       <c r="N262" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="263" spans="1:14" x14ac:dyDescent="0.25">
@@ -42029,7 +42029,7 @@
         <v>0</v>
       </c>
       <c r="N263" s="8">
-        <v>3423</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="264" spans="1:14" x14ac:dyDescent="0.25">
@@ -42073,7 +42073,7 @@
         <v>0</v>
       </c>
       <c r="N264" s="8">
-        <v>10262</v>
+        <v>4512</v>
       </c>
     </row>
     <row r="265" spans="1:14" x14ac:dyDescent="0.25">
@@ -42117,7 +42117,7 @@
         <v>0</v>
       </c>
       <c r="N265" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="266" spans="1:14" x14ac:dyDescent="0.25">
@@ -42161,7 +42161,7 @@
         <v>0</v>
       </c>
       <c r="N266" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="267" spans="1:14" x14ac:dyDescent="0.25">
@@ -42205,7 +42205,7 @@
         <v>0</v>
       </c>
       <c r="N267" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="268" spans="1:14" x14ac:dyDescent="0.25">
@@ -42249,7 +42249,7 @@
         <v>0</v>
       </c>
       <c r="N268" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="269" spans="1:14" x14ac:dyDescent="0.25">
@@ -42293,7 +42293,7 @@
         <v>0</v>
       </c>
       <c r="N269" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="270" spans="1:14" x14ac:dyDescent="0.25">
@@ -42337,7 +42337,7 @@
         <v>0</v>
       </c>
       <c r="N270" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="271" spans="1:14" x14ac:dyDescent="0.25">
@@ -42381,7 +42381,7 @@
         <v>0</v>
       </c>
       <c r="N271" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="272" spans="1:14" x14ac:dyDescent="0.25">
@@ -42425,7 +42425,7 @@
         <v>0</v>
       </c>
       <c r="N272" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="273" spans="1:14" x14ac:dyDescent="0.25">
@@ -42469,7 +42469,7 @@
         <v>0</v>
       </c>
       <c r="N273" s="8">
-        <v>4039</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="274" spans="1:14" x14ac:dyDescent="0.25">
@@ -42513,7 +42513,7 @@
         <v>0</v>
       </c>
       <c r="N274" s="8">
-        <v>12124</v>
+        <v>5328</v>
       </c>
     </row>
     <row r="275" spans="1:14" x14ac:dyDescent="0.25">
@@ -42557,7 +42557,7 @@
         <v>0</v>
       </c>
       <c r="N275" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="276" spans="1:14" x14ac:dyDescent="0.25">
@@ -42601,7 +42601,7 @@
         <v>0</v>
       </c>
       <c r="N276" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="277" spans="1:14" x14ac:dyDescent="0.25">
@@ -42645,7 +42645,7 @@
         <v>0</v>
       </c>
       <c r="N277" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="278" spans="1:14" x14ac:dyDescent="0.25">
@@ -42689,7 +42689,7 @@
         <v>0</v>
       </c>
       <c r="N278" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="279" spans="1:14" x14ac:dyDescent="0.25">
@@ -42733,7 +42733,7 @@
         <v>0</v>
       </c>
       <c r="N279" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="280" spans="1:14" x14ac:dyDescent="0.25">
@@ -42777,7 +42777,7 @@
         <v>0</v>
       </c>
       <c r="N280" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="281" spans="1:14" x14ac:dyDescent="0.25">
@@ -42821,7 +42821,7 @@
         <v>0</v>
       </c>
       <c r="N281" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="282" spans="1:14" x14ac:dyDescent="0.25">
@@ -42865,7 +42865,7 @@
         <v>0</v>
       </c>
       <c r="N282" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="283" spans="1:14" x14ac:dyDescent="0.25">
@@ -42909,7 +42909,7 @@
         <v>0</v>
       </c>
       <c r="N283" s="8">
-        <v>4767</v>
+        <v>2096</v>
       </c>
     </row>
     <row r="284" spans="1:14" x14ac:dyDescent="0.25">
@@ -42953,7 +42953,7 @@
         <v>0</v>
       </c>
       <c r="N284" s="8">
-        <v>14308</v>
+        <v>6288</v>
       </c>
     </row>
     <row r="285" spans="1:14" x14ac:dyDescent="0.25">
@@ -42997,7 +42997,7 @@
         <v>0</v>
       </c>
       <c r="N285" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="286" spans="1:14" x14ac:dyDescent="0.25">
@@ -43041,7 +43041,7 @@
         <v>0</v>
       </c>
       <c r="N286" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="287" spans="1:14" x14ac:dyDescent="0.25">
@@ -43085,7 +43085,7 @@
         <v>0</v>
       </c>
       <c r="N287" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="288" spans="1:14" x14ac:dyDescent="0.25">
@@ -43129,7 +43129,7 @@
         <v>0</v>
       </c>
       <c r="N288" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="289" spans="1:14" x14ac:dyDescent="0.25">
@@ -43173,7 +43173,7 @@
         <v>0</v>
       </c>
       <c r="N289" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="290" spans="1:14" x14ac:dyDescent="0.25">
@@ -43217,7 +43217,7 @@
         <v>0</v>
       </c>
       <c r="N290" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="291" spans="1:14" x14ac:dyDescent="0.25">
@@ -43261,7 +43261,7 @@
         <v>0</v>
       </c>
       <c r="N291" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="292" spans="1:14" x14ac:dyDescent="0.25">
@@ -43305,7 +43305,7 @@
         <v>0</v>
       </c>
       <c r="N292" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="293" spans="1:14" x14ac:dyDescent="0.25">
@@ -43349,7 +43349,7 @@
         <v>0</v>
       </c>
       <c r="N293" s="8">
-        <v>5621</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="294" spans="1:14" x14ac:dyDescent="0.25">
@@ -43393,7 +43393,7 @@
         <v>0</v>
       </c>
       <c r="N294" s="8">
-        <v>16870</v>
+        <v>7416</v>
       </c>
     </row>
     <row r="295" spans="1:14" x14ac:dyDescent="0.25">
@@ -43437,7 +43437,7 @@
         <v>0</v>
       </c>
       <c r="N295" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="296" spans="1:14" x14ac:dyDescent="0.25">
@@ -43481,7 +43481,7 @@
         <v>0</v>
       </c>
       <c r="N296" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="297" spans="1:14" x14ac:dyDescent="0.25">
@@ -43525,7 +43525,7 @@
         <v>0</v>
       </c>
       <c r="N297" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="298" spans="1:14" x14ac:dyDescent="0.25">
@@ -43569,7 +43569,7 @@
         <v>0</v>
       </c>
       <c r="N298" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="299" spans="1:14" x14ac:dyDescent="0.25">
@@ -43613,7 +43613,7 @@
         <v>0</v>
       </c>
       <c r="N299" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="300" spans="1:14" x14ac:dyDescent="0.25">
@@ -43657,7 +43657,7 @@
         <v>0</v>
       </c>
       <c r="N300" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="301" spans="1:14" x14ac:dyDescent="0.25">
@@ -43701,7 +43701,7 @@
         <v>0</v>
       </c>
       <c r="N301" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="302" spans="1:14" x14ac:dyDescent="0.25">
@@ -43745,7 +43745,7 @@
         <v>0</v>
       </c>
       <c r="N302" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="303" spans="1:14" x14ac:dyDescent="0.25">
@@ -43789,7 +43789,7 @@
         <v>0</v>
       </c>
       <c r="N303" s="8">
-        <v>6636</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="304" spans="1:14" x14ac:dyDescent="0.25">
@@ -43833,7 +43833,7 @@
         <v>0</v>
       </c>
       <c r="N304" s="8">
-        <v>19901</v>
+        <v>8748</v>
       </c>
     </row>
   </sheetData>
@@ -53237,7 +53237,7 @@
         <v>24</v>
       </c>
       <c r="E5">
-        <v>5460</v>
+        <v>2400</v>
       </c>
       <c r="F5">
         <v>1500</v>
@@ -53266,7 +53266,7 @@
         <v>49</v>
       </c>
       <c r="E6">
-        <v>9100</v>
+        <v>4000</v>
       </c>
       <c r="F6">
         <v>3000</v>
@@ -53295,7 +53295,7 @@
         <v>99</v>
       </c>
       <c r="E7">
-        <v>15925</v>
+        <v>7000</v>
       </c>
       <c r="F7">
         <v>6000</v>
@@ -53324,7 +53324,7 @@
         <v>199</v>
       </c>
       <c r="E8">
-        <v>27300</v>
+        <v>12000</v>
       </c>
       <c r="F8">
         <v>12000</v>
@@ -53353,7 +53353,7 @@
         <v>299</v>
       </c>
       <c r="E9">
-        <v>45500</v>
+        <v>20000</v>
       </c>
       <c r="F9">
         <v>24000</v>
@@ -53382,7 +53382,7 @@
         <v>999999</v>
       </c>
       <c r="E10">
-        <v>81900</v>
+        <v>36000</v>
       </c>
       <c r="F10">
         <v>43200</v>
@@ -53406,7 +53406,7 @@
   <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E1" t="s">
         <v>1222</v>
       </c>

</xml_diff>

<commit_message>
chore: prepare v0.5.0 release
Everything accumulated in [Unreleased] since v0.2.0 (informally labeled
v0.3.0/v0.4.0 in individual CHANGELOG bullets and PatchNoteTable rows along
the way, but never actually tagged/released as such) ships together as
v0.5.0: data-table balance rework, exist tree 250 nodes, 300 stages, 150
weapons, ranking, sound, bulk actions, multi-crit, and several rounds of
reward/difficulty rebalancing.

- CHANGELOG.md: moved [Unreleased] into ## [v0.5.0] - 2026-09-13, added a
  short summary paragraph, left a fresh empty [Unreleased] above it.
- PatchNoteTable: consolidated all v0.3.0/v0.4.0 rows into v0.5.0 (27 rows,
  SortOrder renumbered 1-27, ReleaseDate set to 2026-09-13).
- SAVE_VERSION bumped 6 -> 7 per docs/RELEASE.md 3절 (mandatory on every
  release regardless of save-shape changes).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5770" uniqueCount="1427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5770" uniqueCount="1426">
   <si>
     <t>enum 그룹</t>
   </si>
@@ -4293,13 +4293,10 @@
     <t>2026-09-11</t>
   </si>
   <si>
-    <t>v0.3.0</t>
-  </si>
-  <si>
-    <t>v0.4.0</t>
-  </si>
-  <si>
-    <t>2026-09-12</t>
+    <t>v0.5.0</t>
+  </si>
+  <si>
+    <t>2026-09-13</t>
   </si>
   <si>
     <t>해금 조건(존재력 트리 해금 수)</t>
@@ -16337,7 +16334,7 @@
         <v>1167</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>1171</v>
@@ -16355,7 +16352,7 @@
         <v>1179</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>1181</v>
@@ -16373,7 +16370,7 @@
         <v>1189</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -16455,7 +16452,7 @@
         <v>1180</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="K4" s="12" t="s">
         <v>1182</v>
@@ -16910,7 +16907,7 @@
         <v>1205</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -53509,7 +53506,7 @@
   <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="17.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.4" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E1" t="s">
         <v>1235</v>
       </c>
@@ -53850,7 +53847,7 @@
         <v>1419</v>
       </c>
       <c r="D16" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E16" t="s">
         <v>94</v>
@@ -53873,7 +53870,7 @@
         <v>1419</v>
       </c>
       <c r="D17" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E17" t="s">
         <v>94</v>
@@ -53896,7 +53893,7 @@
         <v>1419</v>
       </c>
       <c r="D18" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E18" t="s">
         <v>94</v>
@@ -53919,7 +53916,7 @@
         <v>1419</v>
       </c>
       <c r="D19" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E19" t="s">
         <v>91</v>
@@ -53942,7 +53939,7 @@
         <v>1419</v>
       </c>
       <c r="D20" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E20" t="s">
         <v>91</v>
@@ -53965,7 +53962,7 @@
         <v>1419</v>
       </c>
       <c r="D21" t="s">
-        <v>1418</v>
+        <v>1420</v>
       </c>
       <c r="E21" t="s">
         <v>94</v>
@@ -53985,10 +53982,10 @@
         <v>33018</v>
       </c>
       <c r="C22" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D22" t="s">
         <v>1420</v>
-      </c>
-      <c r="D22" t="s">
-        <v>1421</v>
       </c>
       <c r="E22" t="s">
         <v>91</v>
@@ -53997,7 +53994,7 @@
         <v>55020</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -54008,10 +54005,10 @@
         <v>33019</v>
       </c>
       <c r="C23" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D23" t="s">
         <v>1420</v>
-      </c>
-      <c r="D23" t="s">
-        <v>1421</v>
       </c>
       <c r="E23" t="s">
         <v>94</v>
@@ -54020,7 +54017,7 @@
         <v>55024</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -54031,10 +54028,10 @@
         <v>33020</v>
       </c>
       <c r="C24" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D24" t="s">
         <v>1420</v>
-      </c>
-      <c r="D24" t="s">
-        <v>1421</v>
       </c>
       <c r="E24" t="s">
         <v>96</v>
@@ -54043,7 +54040,7 @@
         <v>55026</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -54054,10 +54051,10 @@
         <v>33021</v>
       </c>
       <c r="C25" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D25" t="s">
         <v>1420</v>
-      </c>
-      <c r="D25" t="s">
-        <v>1421</v>
       </c>
       <c r="E25" t="s">
         <v>91</v>
@@ -54066,7 +54063,7 @@
         <v>55027</v>
       </c>
       <c r="G25">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -54077,10 +54074,10 @@
         <v>33022</v>
       </c>
       <c r="C26" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D26" t="s">
         <v>1420</v>
-      </c>
-      <c r="D26" t="s">
-        <v>1421</v>
       </c>
       <c r="E26" t="s">
         <v>91</v>
@@ -54089,7 +54086,7 @@
         <v>55028</v>
       </c>
       <c r="G26">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -54100,10 +54097,10 @@
         <v>33023</v>
       </c>
       <c r="C27" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D27" t="s">
         <v>1420</v>
-      </c>
-      <c r="D27" t="s">
-        <v>1421</v>
       </c>
       <c r="E27" t="s">
         <v>91</v>
@@ -54112,7 +54109,7 @@
         <v>55029</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -54123,10 +54120,10 @@
         <v>33024</v>
       </c>
       <c r="C28" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D28" t="s">
         <v>1420</v>
-      </c>
-      <c r="D28" t="s">
-        <v>1421</v>
       </c>
       <c r="E28" t="s">
         <v>96</v>
@@ -54135,7 +54132,7 @@
         <v>55030</v>
       </c>
       <c r="G28">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -54146,10 +54143,10 @@
         <v>33025</v>
       </c>
       <c r="C29" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D29" t="s">
         <v>1420</v>
-      </c>
-      <c r="D29" t="s">
-        <v>1421</v>
       </c>
       <c r="E29" t="s">
         <v>94</v>
@@ -54158,7 +54155,7 @@
         <v>55031</v>
       </c>
       <c r="G29">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -54169,10 +54166,10 @@
         <v>33026</v>
       </c>
       <c r="C30" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D30" t="s">
         <v>1420</v>
-      </c>
-      <c r="D30" t="s">
-        <v>1421</v>
       </c>
       <c r="E30" t="s">
         <v>91</v>
@@ -54181,7 +54178,7 @@
         <v>55032</v>
       </c>
       <c r="G30">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -54192,10 +54189,10 @@
         <v>33027</v>
       </c>
       <c r="C31" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D31" t="s">
         <v>1420</v>
-      </c>
-      <c r="D31" t="s">
-        <v>1421</v>
       </c>
       <c r="E31" t="s">
         <v>91</v>
@@ -54204,7 +54201,7 @@
         <v>55033</v>
       </c>
       <c r="G31">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -54215,10 +54212,10 @@
         <v>33028</v>
       </c>
       <c r="C32" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D32" t="s">
         <v>1420</v>
-      </c>
-      <c r="D32" t="s">
-        <v>1421</v>
       </c>
       <c r="E32" t="s">
         <v>94</v>
@@ -54227,7 +54224,7 @@
         <v>55034</v>
       </c>
       <c r="G32">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
@@ -54238,10 +54235,10 @@
         <v>33029</v>
       </c>
       <c r="C33" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D33" t="s">
         <v>1420</v>
-      </c>
-      <c r="D33" t="s">
-        <v>1421</v>
       </c>
       <c r="E33" t="s">
         <v>94</v>
@@ -54250,7 +54247,7 @@
         <v>55035</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -54261,10 +54258,10 @@
         <v>33030</v>
       </c>
       <c r="C34" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D34" t="s">
         <v>1420</v>
-      </c>
-      <c r="D34" t="s">
-        <v>1421</v>
       </c>
       <c r="E34" t="s">
         <v>91</v>
@@ -54273,7 +54270,7 @@
         <v>55036</v>
       </c>
       <c r="G34">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
@@ -54284,10 +54281,10 @@
         <v>33031</v>
       </c>
       <c r="C35" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D35" t="s">
         <v>1420</v>
-      </c>
-      <c r="D35" t="s">
-        <v>1421</v>
       </c>
       <c r="E35" t="s">
         <v>94</v>
@@ -54296,7 +54293,7 @@
         <v>55037</v>
       </c>
       <c r="G35">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -54307,10 +54304,10 @@
         <v>33032</v>
       </c>
       <c r="C36" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D36" t="s">
         <v>1420</v>
-      </c>
-      <c r="D36" t="s">
-        <v>1421</v>
       </c>
       <c r="E36" t="s">
         <v>91</v>
@@ -54319,7 +54316,7 @@
         <v>55038</v>
       </c>
       <c r="G36">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
@@ -54330,10 +54327,10 @@
         <v>33033</v>
       </c>
       <c r="C37" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D37" t="s">
         <v>1420</v>
-      </c>
-      <c r="D37" t="s">
-        <v>1421</v>
       </c>
       <c r="E37" t="s">
         <v>91</v>
@@ -54342,7 +54339,7 @@
         <v>55039</v>
       </c>
       <c r="G37">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
@@ -54353,10 +54350,10 @@
         <v>33034</v>
       </c>
       <c r="C38" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D38" t="s">
         <v>1420</v>
-      </c>
-      <c r="D38" t="s">
-        <v>1421</v>
       </c>
       <c r="E38" t="s">
         <v>91</v>
@@ -54365,7 +54362,7 @@
         <v>55040</v>
       </c>
       <c r="G38">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
@@ -54376,10 +54373,10 @@
         <v>33035</v>
       </c>
       <c r="C39" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D39" t="s">
         <v>1420</v>
-      </c>
-      <c r="D39" t="s">
-        <v>1421</v>
       </c>
       <c r="E39" t="s">
         <v>94</v>
@@ -54388,7 +54385,7 @@
         <v>55041</v>
       </c>
       <c r="G39">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
@@ -54399,10 +54396,10 @@
         <v>33036</v>
       </c>
       <c r="C40" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D40" t="s">
         <v>1420</v>
-      </c>
-      <c r="D40" t="s">
-        <v>1421</v>
       </c>
       <c r="E40" t="s">
         <v>94</v>
@@ -54411,7 +54408,7 @@
         <v>55042</v>
       </c>
       <c r="G40">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
@@ -54422,10 +54419,10 @@
         <v>33037</v>
       </c>
       <c r="C41" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D41" t="s">
         <v>1420</v>
-      </c>
-      <c r="D41" t="s">
-        <v>1421</v>
       </c>
       <c r="E41" t="s">
         <v>94</v>
@@ -54434,7 +54431,7 @@
         <v>55043</v>
       </c>
       <c r="G41">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
@@ -54445,10 +54442,10 @@
         <v>33038</v>
       </c>
       <c r="C42" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D42" t="s">
         <v>1420</v>
-      </c>
-      <c r="D42" t="s">
-        <v>1421</v>
       </c>
       <c r="E42" t="s">
         <v>94</v>
@@ -54457,7 +54454,7 @@
         <v>55044</v>
       </c>
       <c r="G42">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
balance: 활/도끼 및 치명타(CRIT/CRIT_DMG) 획득량 하향
- 활(치확 특화)·도끼(치피 특화) WeaponTable 보유/장착 효과 하향 — 검/창은
  PrimaryStat이 달라 스키마상 자동으로 대상에서 빠짐
- CRIT 획득량 절반, CRIT_DMG 획득량 10분의 1로 하향(StatTable/
  ExistTreeTable/WeaponTable/RelicTable 전반). 깡스탯×퍼센트 곱연산
  구조에서 두 원천에 목표 배율을 그대로 곱하면 결과가 제곱으로 깎이는
  것을 확인해, 목표 배율의 제곱근을 각 원천에 곱하는 방식으로 보정
- CRIT_DMG의 StatTable 기본값(150)은 유지 — 치확 낮은 구간에서 크리티컬이
  논크리티컬보다 약해지는 모순을 방지
- 검증: 무기 종류별 동일 투자 시 DPS 비교, 존재력 트리만으로 치확
  100%/200% 도달 시점 비교 — 자세한 내용은 CHANGELOG.md 참고

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/balance/balance.xlsx
+++ b/balance/balance.xlsx
@@ -10572,10 +10572,10 @@
         <v>0.5</v>
       </c>
       <c r="M55" s="8">
-        <v>1</v>
+        <v>0.707107</v>
       </c>
       <c r="N55" s="8">
-        <v>3</v>
+        <v>2.12132</v>
       </c>
       <c r="O55" s="1" t="s">
         <v>1255</v>
@@ -10622,10 +10622,10 @@
         <v>0.55</v>
       </c>
       <c r="M56" s="8">
-        <v>1.1</v>
+        <v>0.777817</v>
       </c>
       <c r="N56" s="8">
-        <v>3.3</v>
+        <v>2.333452</v>
       </c>
       <c r="O56" s="1" t="s">
         <v>1255</v>
@@ -10672,10 +10672,10 @@
         <v>0.6</v>
       </c>
       <c r="M57" s="8">
-        <v>1.21</v>
+        <v>0.855599</v>
       </c>
       <c r="N57" s="8">
-        <v>3.6</v>
+        <v>2.545584</v>
       </c>
       <c r="O57" s="1" t="s">
         <v>1255</v>
@@ -10722,10 +10722,10 @@
         <v>0.65</v>
       </c>
       <c r="M58" s="8">
-        <v>1.33</v>
+        <v>0.940452</v>
       </c>
       <c r="N58" s="8">
-        <v>3.9</v>
+        <v>2.757716</v>
       </c>
       <c r="O58" s="1" t="s">
         <v>1255</v>
@@ -10772,10 +10772,10 @@
         <v>0.7</v>
       </c>
       <c r="M59" s="8">
-        <v>1.46</v>
+        <v>1.032376</v>
       </c>
       <c r="N59" s="8">
-        <v>4.2</v>
+        <v>2.969848</v>
       </c>
       <c r="O59" s="1" t="s">
         <v>1255</v>
@@ -10822,10 +10822,10 @@
         <v>1</v>
       </c>
       <c r="M60" s="8">
-        <v>2</v>
+        <v>1.414214</v>
       </c>
       <c r="N60" s="8">
-        <v>6</v>
+        <v>4.242641</v>
       </c>
       <c r="O60" s="1" t="s">
         <v>1256</v>
@@ -10872,10 +10872,10 @@
         <v>1.1</v>
       </c>
       <c r="M61" s="8">
-        <v>2.2</v>
+        <v>1.555635</v>
       </c>
       <c r="N61" s="8">
-        <v>6.6</v>
+        <v>4.666905</v>
       </c>
       <c r="O61" s="1" t="s">
         <v>1256</v>
@@ -10922,10 +10922,10 @@
         <v>1.2</v>
       </c>
       <c r="M62" s="8">
-        <v>2.42</v>
+        <v>1.711198</v>
       </c>
       <c r="N62" s="8">
-        <v>7.2</v>
+        <v>5.091169</v>
       </c>
       <c r="O62" s="1" t="s">
         <v>1256</v>
@@ -10972,10 +10972,10 @@
         <v>1.3</v>
       </c>
       <c r="M63" s="8">
-        <v>2.66</v>
+        <v>1.880904</v>
       </c>
       <c r="N63" s="8">
-        <v>7.8</v>
+        <v>5.515433</v>
       </c>
       <c r="O63" s="1" t="s">
         <v>1256</v>
@@ -11022,10 +11022,10 @@
         <v>1.4</v>
       </c>
       <c r="M64" s="8">
-        <v>2.93</v>
+        <v>2.071823</v>
       </c>
       <c r="N64" s="8">
-        <v>8.4</v>
+        <v>5.939697</v>
       </c>
       <c r="O64" s="1" t="s">
         <v>1256</v>
@@ -11072,10 +11072,10 @@
         <v>2</v>
       </c>
       <c r="M65" s="8">
-        <v>4</v>
+        <v>2.828427</v>
       </c>
       <c r="N65" s="8">
-        <v>12</v>
+        <v>8.485281</v>
       </c>
       <c r="O65" s="1" t="s">
         <v>1257</v>
@@ -11122,10 +11122,10 @@
         <v>2.2</v>
       </c>
       <c r="M66" s="8">
-        <v>4.4</v>
+        <v>3.11127</v>
       </c>
       <c r="N66" s="8">
-        <v>13.2</v>
+        <v>9.33381</v>
       </c>
       <c r="O66" s="1" t="s">
         <v>1257</v>
@@ -11172,10 +11172,10 @@
         <v>2.4</v>
       </c>
       <c r="M67" s="8">
-        <v>4.84</v>
+        <v>3.422397</v>
       </c>
       <c r="N67" s="8">
-        <v>14.4</v>
+        <v>10.182338</v>
       </c>
       <c r="O67" s="1" t="s">
         <v>1257</v>
@@ -11222,10 +11222,10 @@
         <v>2.6</v>
       </c>
       <c r="M68" s="8">
-        <v>5.32</v>
+        <v>3.761808</v>
       </c>
       <c r="N68" s="8">
-        <v>15.6</v>
+        <v>11.030866</v>
       </c>
       <c r="O68" s="1" t="s">
         <v>1257</v>
@@ -11272,10 +11272,10 @@
         <v>2.8</v>
       </c>
       <c r="M69" s="8">
-        <v>5.86</v>
+        <v>4.143646</v>
       </c>
       <c r="N69" s="8">
-        <v>16.8</v>
+        <v>11.879394</v>
       </c>
       <c r="O69" s="1" t="s">
         <v>1257</v>
@@ -11322,10 +11322,10 @@
         <v>4</v>
       </c>
       <c r="M70" s="8">
-        <v>8</v>
+        <v>5.656854</v>
       </c>
       <c r="N70" s="8">
-        <v>24</v>
+        <v>16.970563</v>
       </c>
       <c r="O70" s="1" t="s">
         <v>1258</v>
@@ -11372,10 +11372,10 @@
         <v>4.4</v>
       </c>
       <c r="M71" s="8">
-        <v>8.8</v>
+        <v>6.22254</v>
       </c>
       <c r="N71" s="8">
-        <v>26.4</v>
+        <v>18.667619</v>
       </c>
       <c r="O71" s="1" t="s">
         <v>1258</v>
@@ -11422,10 +11422,10 @@
         <v>4.8</v>
       </c>
       <c r="M72" s="8">
-        <v>9.68</v>
+        <v>6.844794</v>
       </c>
       <c r="N72" s="8">
-        <v>28.8</v>
+        <v>20.364675</v>
       </c>
       <c r="O72" s="1" t="s">
         <v>1258</v>
@@ -11472,10 +11472,10 @@
         <v>5.2</v>
       </c>
       <c r="M73" s="8">
-        <v>10.65</v>
+        <v>7.530687</v>
       </c>
       <c r="N73" s="8">
-        <v>31.2</v>
+        <v>22.061732</v>
       </c>
       <c r="O73" s="1" t="s">
         <v>1258</v>
@@ -11522,10 +11522,10 @@
         <v>5.6</v>
       </c>
       <c r="M74" s="8">
-        <v>11.71</v>
+        <v>8.28022</v>
       </c>
       <c r="N74" s="8">
-        <v>33.6</v>
+        <v>23.758788</v>
       </c>
       <c r="O74" s="1" t="s">
         <v>1258</v>
@@ -11572,10 +11572,10 @@
         <v>8</v>
       </c>
       <c r="M75" s="8">
-        <v>16</v>
+        <v>11.313708</v>
       </c>
       <c r="N75" s="8">
-        <v>48</v>
+        <v>33.941125</v>
       </c>
       <c r="O75" s="1" t="s">
         <v>1259</v>
@@ -11622,10 +11622,10 @@
         <v>8.8</v>
       </c>
       <c r="M76" s="8">
-        <v>17.6</v>
+        <v>12.445079</v>
       </c>
       <c r="N76" s="8">
-        <v>52.8</v>
+        <v>37.335238</v>
       </c>
       <c r="O76" s="1" t="s">
         <v>1259</v>
@@ -11672,10 +11672,10 @@
         <v>9.6</v>
       </c>
       <c r="M77" s="8">
-        <v>19.36</v>
+        <v>13.689587</v>
       </c>
       <c r="N77" s="8">
-        <v>57.6</v>
+        <v>40.729351</v>
       </c>
       <c r="O77" s="1" t="s">
         <v>1259</v>
@@ -11722,10 +11722,10 @@
         <v>10.4</v>
       </c>
       <c r="M78" s="8">
-        <v>21.3</v>
+        <v>15.061374</v>
       </c>
       <c r="N78" s="8">
-        <v>62.4</v>
+        <v>44.123463</v>
       </c>
       <c r="O78" s="1" t="s">
         <v>1259</v>
@@ -11772,10 +11772,10 @@
         <v>11.2</v>
       </c>
       <c r="M79" s="8">
-        <v>23.43</v>
+        <v>16.567512</v>
       </c>
       <c r="N79" s="8">
-        <v>67.2</v>
+        <v>47.517576</v>
       </c>
       <c r="O79" s="1" t="s">
         <v>1259</v>
@@ -12302,10 +12302,10 @@
         <v>16</v>
       </c>
       <c r="M90" s="8">
-        <v>32</v>
+        <v>22.627417</v>
       </c>
       <c r="N90" s="8">
-        <v>96</v>
+        <v>67.882251</v>
       </c>
       <c r="O90" s="1" t="s">
         <v>1260</v>
@@ -12350,10 +12350,10 @@
         <v>17.6</v>
       </c>
       <c r="M91" s="8">
-        <v>35.2</v>
+        <v>24.890159</v>
       </c>
       <c r="N91" s="8">
-        <v>105.6</v>
+        <v>74.670476</v>
       </c>
       <c r="O91" s="1" t="s">
         <v>1260</v>
@@ -12398,10 +12398,10 @@
         <v>19.2</v>
       </c>
       <c r="M92" s="8">
-        <v>38.72</v>
+        <v>27.379175</v>
       </c>
       <c r="N92" s="8">
-        <v>115.2</v>
+        <v>81.458701</v>
       </c>
       <c r="O92" s="1" t="s">
         <v>1260</v>
@@ -12446,10 +12446,10 @@
         <v>20.8</v>
       </c>
       <c r="M93" s="8">
-        <v>42.592</v>
+        <v>30.117092</v>
       </c>
       <c r="N93" s="8">
-        <v>124.8</v>
+        <v>88.246926</v>
       </c>
       <c r="O93" s="1" t="s">
         <v>1260</v>
@@ -12494,10 +12494,10 @@
         <v>22.4</v>
       </c>
       <c r="M94" s="8">
-        <v>46.851</v>
+        <v>33.12866</v>
       </c>
       <c r="N94" s="8">
-        <v>134.4</v>
+        <v>95.035151</v>
       </c>
       <c r="O94" s="1" t="s">
         <v>1260</v>
@@ -12542,10 +12542,10 @@
         <v>0.5</v>
       </c>
       <c r="M95" s="8">
-        <v>1</v>
+        <v>0.316228</v>
       </c>
       <c r="N95" s="8">
-        <v>10</v>
+        <v>3.162278</v>
       </c>
       <c r="O95" s="1" t="s">
         <v>1255</v>
@@ -12590,10 +12590,10 @@
         <v>0.55</v>
       </c>
       <c r="M96" s="8">
-        <v>1.1</v>
+        <v>0.347851</v>
       </c>
       <c r="N96" s="8">
-        <v>11</v>
+        <v>3.478505</v>
       </c>
       <c r="O96" s="1" t="s">
         <v>1255</v>
@@ -12638,10 +12638,10 @@
         <v>0.6</v>
       </c>
       <c r="M97" s="8">
-        <v>1.21</v>
+        <v>0.382636</v>
       </c>
       <c r="N97" s="8">
-        <v>12</v>
+        <v>3.794733</v>
       </c>
       <c r="O97" s="1" t="s">
         <v>1255</v>
@@ -12686,10 +12686,10 @@
         <v>0.65</v>
       </c>
       <c r="M98" s="8">
-        <v>1.331</v>
+        <v>0.420899</v>
       </c>
       <c r="N98" s="8">
-        <v>13</v>
+        <v>4.110961</v>
       </c>
       <c r="O98" s="1" t="s">
         <v>1255</v>
@@ -12734,10 +12734,10 @@
         <v>0.7</v>
       </c>
       <c r="M99" s="8">
-        <v>1.464</v>
+        <v>0.462957</v>
       </c>
       <c r="N99" s="8">
-        <v>14</v>
+        <v>4.427189</v>
       </c>
       <c r="O99" s="1" t="s">
         <v>1255</v>
@@ -12782,10 +12782,10 @@
         <v>1</v>
       </c>
       <c r="M100" s="8">
-        <v>2</v>
+        <v>0.632456</v>
       </c>
       <c r="N100" s="8">
-        <v>20</v>
+        <v>6.324555</v>
       </c>
       <c r="O100" s="1" t="s">
         <v>1256</v>
@@ -12830,10 +12830,10 @@
         <v>1.1</v>
       </c>
       <c r="M101" s="8">
-        <v>2.2</v>
+        <v>0.695701</v>
       </c>
       <c r="N101" s="8">
-        <v>22</v>
+        <v>6.957011</v>
       </c>
       <c r="O101" s="1" t="s">
         <v>1256</v>
@@ -12878,10 +12878,10 @@
         <v>1.2</v>
       </c>
       <c r="M102" s="8">
-        <v>2.42</v>
+        <v>0.765271</v>
       </c>
       <c r="N102" s="8">
-        <v>24</v>
+        <v>7.589466</v>
       </c>
       <c r="O102" s="1" t="s">
         <v>1256</v>
@@ -12926,10 +12926,10 @@
         <v>1.3</v>
       </c>
       <c r="M103" s="8">
-        <v>2.662</v>
+        <v>0.841798</v>
       </c>
       <c r="N103" s="8">
-        <v>26</v>
+        <v>8.221922</v>
       </c>
       <c r="O103" s="1" t="s">
         <v>1256</v>
@@ -12974,10 +12974,10 @@
         <v>1.4</v>
       </c>
       <c r="M104" s="8">
-        <v>2.928</v>
+        <v>0.925915</v>
       </c>
       <c r="N104" s="8">
-        <v>28</v>
+        <v>8.854377</v>
       </c>
       <c r="O104" s="1" t="s">
         <v>1256</v>
@@ -13022,10 +13022,10 @@
         <v>2</v>
       </c>
       <c r="M105" s="8">
-        <v>4</v>
+        <v>1.264911</v>
       </c>
       <c r="N105" s="8">
-        <v>40</v>
+        <v>12.649111</v>
       </c>
       <c r="O105" s="1" t="s">
         <v>1257</v>
@@ -13070,10 +13070,10 @@
         <v>2.2</v>
       </c>
       <c r="M106" s="8">
-        <v>4.4</v>
+        <v>1.391402</v>
       </c>
       <c r="N106" s="8">
-        <v>44</v>
+        <v>13.914022</v>
       </c>
       <c r="O106" s="1" t="s">
         <v>1257</v>
@@ -13118,10 +13118,10 @@
         <v>2.4</v>
       </c>
       <c r="M107" s="8">
-        <v>4.84</v>
+        <v>1.530542</v>
       </c>
       <c r="N107" s="8">
-        <v>48</v>
+        <v>15.178933</v>
       </c>
       <c r="O107" s="1" t="s">
         <v>1257</v>
@@ -13166,10 +13166,10 @@
         <v>2.6</v>
       </c>
       <c r="M108" s="8">
-        <v>5.324</v>
+        <v>1.683597</v>
       </c>
       <c r="N108" s="8">
-        <v>52</v>
+        <v>16.443844</v>
       </c>
       <c r="O108" s="1" t="s">
         <v>1257</v>
@@ -13214,10 +13214,10 @@
         <v>2.8</v>
       </c>
       <c r="M109" s="8">
-        <v>5.856</v>
+        <v>1.85183</v>
       </c>
       <c r="N109" s="8">
-        <v>56</v>
+        <v>17.708755</v>
       </c>
       <c r="O109" s="1" t="s">
         <v>1257</v>
@@ -13262,10 +13262,10 @@
         <v>4</v>
       </c>
       <c r="M110" s="8">
-        <v>8</v>
+        <v>2.529822</v>
       </c>
       <c r="N110" s="8">
-        <v>80</v>
+        <v>25.298221</v>
       </c>
       <c r="O110" s="1" t="s">
         <v>1258</v>
@@ -13310,10 +13310,10 @@
         <v>4.4</v>
       </c>
       <c r="M111" s="8">
-        <v>8.8</v>
+        <v>2.782804</v>
       </c>
       <c r="N111" s="8">
-        <v>88</v>
+        <v>27.828043</v>
       </c>
       <c r="O111" s="1" t="s">
         <v>1258</v>
@@ -13358,10 +13358,10 @@
         <v>4.8</v>
       </c>
       <c r="M112" s="8">
-        <v>9.68</v>
+        <v>3.061085</v>
       </c>
       <c r="N112" s="8">
-        <v>96</v>
+        <v>30.357866</v>
       </c>
       <c r="O112" s="1" t="s">
         <v>1258</v>
@@ -13406,10 +13406,10 @@
         <v>5.2</v>
       </c>
       <c r="M113" s="8">
-        <v>10.648</v>
+        <v>3.367193</v>
       </c>
       <c r="N113" s="8">
-        <v>104</v>
+        <v>32.887688</v>
       </c>
       <c r="O113" s="1" t="s">
         <v>1258</v>
@@ -13454,10 +13454,10 @@
         <v>5.6</v>
       </c>
       <c r="M114" s="8">
-        <v>11.713</v>
+        <v>3.703976</v>
       </c>
       <c r="N114" s="8">
-        <v>112</v>
+        <v>35.41751</v>
       </c>
       <c r="O114" s="1" t="s">
         <v>1258</v>
@@ -13502,10 +13502,10 @@
         <v>8</v>
       </c>
       <c r="M115" s="8">
-        <v>16</v>
+        <v>5.059644</v>
       </c>
       <c r="N115" s="8">
-        <v>160</v>
+        <v>50.596443</v>
       </c>
       <c r="O115" s="1" t="s">
         <v>1259</v>
@@ -13550,10 +13550,10 @@
         <v>8.8</v>
       </c>
       <c r="M116" s="8">
-        <v>17.6</v>
+        <v>5.565609</v>
       </c>
       <c r="N116" s="8">
-        <v>176</v>
+        <v>55.656087</v>
       </c>
       <c r="O116" s="1" t="s">
         <v>1259</v>
@@ -13598,10 +13598,10 @@
         <v>9.6</v>
       </c>
       <c r="M117" s="8">
-        <v>19.36</v>
+        <v>6.12217</v>
       </c>
       <c r="N117" s="8">
-        <v>192</v>
+        <v>60.715731</v>
       </c>
       <c r="O117" s="1" t="s">
         <v>1259</v>
@@ -13646,10 +13646,10 @@
         <v>10.4</v>
       </c>
       <c r="M118" s="8">
-        <v>21.296</v>
+        <v>6.734387</v>
       </c>
       <c r="N118" s="8">
-        <v>208</v>
+        <v>65.775375</v>
       </c>
       <c r="O118" s="1" t="s">
         <v>1259</v>
@@ -13694,10 +13694,10 @@
         <v>11.2</v>
       </c>
       <c r="M119" s="8">
-        <v>23.426</v>
+        <v>7.407952</v>
       </c>
       <c r="N119" s="8">
-        <v>224</v>
+        <v>70.83502</v>
       </c>
       <c r="O119" s="1" t="s">
         <v>1259</v>
@@ -13742,10 +13742,10 @@
         <v>16</v>
       </c>
       <c r="M120" s="8">
-        <v>32</v>
+        <v>10.119289</v>
       </c>
       <c r="N120" s="8">
-        <v>320</v>
+        <v>101.192885</v>
       </c>
       <c r="O120" s="1" t="s">
         <v>1260</v>
@@ -13790,10 +13790,10 @@
         <v>17.6</v>
       </c>
       <c r="M121" s="8">
-        <v>35.2</v>
+        <v>11.131217</v>
       </c>
       <c r="N121" s="8">
-        <v>352</v>
+        <v>111.312174</v>
       </c>
       <c r="O121" s="1" t="s">
         <v>1260</v>
@@ -13838,10 +13838,10 @@
         <v>19.2</v>
       </c>
       <c r="M122" s="8">
-        <v>38.72</v>
+        <v>12.244339</v>
       </c>
       <c r="N122" s="8">
-        <v>384</v>
+        <v>121.431462</v>
       </c>
       <c r="O122" s="1" t="s">
         <v>1260</v>
@@ -13886,10 +13886,10 @@
         <v>20.8</v>
       </c>
       <c r="M123" s="8">
-        <v>42.592</v>
+        <v>13.468773</v>
       </c>
       <c r="N123" s="8">
-        <v>416</v>
+        <v>131.550751</v>
       </c>
       <c r="O123" s="1" t="s">
         <v>1260</v>
@@ -13934,10 +13934,10 @@
         <v>22.4</v>
       </c>
       <c r="M124" s="8">
-        <v>46.851</v>
+        <v>14.815587</v>
       </c>
       <c r="N124" s="8">
-        <v>448</v>
+        <v>141.670039</v>
       </c>
       <c r="O124" s="1" t="s">
         <v>1260</v>
@@ -15825,7 +15825,7 @@
         <v>71</v>
       </c>
       <c r="I7" s="8">
-        <v>2</v>
+        <v>1.414214</v>
       </c>
       <c r="J7" s="8">
         <v>20</v>
@@ -15901,7 +15901,7 @@
         <v>72</v>
       </c>
       <c r="I9" s="8">
-        <v>15</v>
+        <v>4.743416</v>
       </c>
       <c r="J9" s="8">
         <v>30</v>
@@ -16167,7 +16167,7 @@
         <v>72</v>
       </c>
       <c r="I16">
-        <v>18</v>
+        <v>5.6921</v>
       </c>
       <c r="J16">
         <v>10</v>
@@ -44187,7 +44187,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="8">
-        <v>0.5</v>
+        <v>0.353553</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>1095</v>
@@ -44219,7 +44219,7 @@
         <v>150</v>
       </c>
       <c r="G8" s="8">
-        <v>2</v>
+        <v>0.632456</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>1095</v>
@@ -44685,7 +44685,7 @@
         <v>185</v>
       </c>
       <c r="J12" s="8">
-        <v>5</v>
+        <v>3.535534</v>
       </c>
       <c r="K12" s="8">
         <v>31</v>
@@ -44720,7 +44720,7 @@
         <v>185</v>
       </c>
       <c r="J13" s="8">
-        <v>6</v>
+        <v>4.242641</v>
       </c>
       <c r="K13" s="8">
         <v>35</v>
@@ -44755,7 +44755,7 @@
         <v>185</v>
       </c>
       <c r="J14" s="8">
-        <v>7</v>
+        <v>4.949747</v>
       </c>
       <c r="K14" s="8">
         <v>40</v>
@@ -45140,7 +45140,7 @@
         <v>185</v>
       </c>
       <c r="J25" s="8">
-        <v>5</v>
+        <v>1.581139</v>
       </c>
       <c r="K25" s="8">
         <v>186</v>
@@ -45175,7 +45175,7 @@
         <v>185</v>
       </c>
       <c r="J26" s="8">
-        <v>6</v>
+        <v>1.897367</v>
       </c>
       <c r="K26" s="8">
         <v>212</v>
@@ -45210,7 +45210,7 @@
         <v>185</v>
       </c>
       <c r="J27" s="8">
-        <v>7</v>
+        <v>2.213594</v>
       </c>
       <c r="K27" s="8">
         <v>244</v>
@@ -45245,7 +45245,7 @@
         <v>185</v>
       </c>
       <c r="J28" s="8">
-        <v>8</v>
+        <v>2.529822</v>
       </c>
       <c r="K28" s="8">
         <v>280</v>
@@ -45280,7 +45280,7 @@
         <v>185</v>
       </c>
       <c r="J29" s="8">
-        <v>9</v>
+        <v>2.84605</v>
       </c>
       <c r="K29" s="8">
         <v>322</v>
@@ -45315,7 +45315,7 @@
         <v>185</v>
       </c>
       <c r="J30" s="8">
-        <v>10</v>
+        <v>3.162278</v>
       </c>
       <c r="K30" s="8">
         <v>369</v>
@@ -46419,7 +46419,7 @@
       </c>
       <c r="I62" s="1"/>
       <c r="J62" s="8">
-        <v>25</v>
+        <v>7.905694</v>
       </c>
       <c r="K62" s="8">
         <v>25719</v>
@@ -46452,7 +46452,7 @@
       </c>
       <c r="I63" s="1"/>
       <c r="J63" s="8">
-        <v>25.4</v>
+        <v>8.032185</v>
       </c>
       <c r="K63" s="8">
         <v>28877</v>
@@ -46485,7 +46485,7 @@
       </c>
       <c r="I64" s="1"/>
       <c r="J64" s="8">
-        <v>25.8</v>
+        <v>8.158676</v>
       </c>
       <c r="K64" s="8">
         <v>32399</v>
@@ -46518,7 +46518,7 @@
       </c>
       <c r="I65" s="1"/>
       <c r="J65" s="8">
-        <v>25</v>
+        <v>17.67767</v>
       </c>
       <c r="K65" s="8">
         <v>36325</v>
@@ -46551,7 +46551,7 @@
       </c>
       <c r="I66" s="1"/>
       <c r="J66" s="8">
-        <v>25.4</v>
+        <v>17.960512</v>
       </c>
       <c r="K66" s="8">
         <v>40698</v>
@@ -46584,7 +46584,7 @@
       </c>
       <c r="I67" s="1"/>
       <c r="J67" s="8">
-        <v>25.8</v>
+        <v>18.243355</v>
       </c>
       <c r="K67" s="8">
         <v>45565</v>
@@ -46617,7 +46617,7 @@
       </c>
       <c r="I68" s="1"/>
       <c r="J68" s="8">
-        <v>26.2</v>
+        <v>18.526198</v>
       </c>
       <c r="K68" s="8">
         <v>50978</v>
@@ -46650,7 +46650,7 @@
       </c>
       <c r="I69" s="1"/>
       <c r="J69" s="8">
-        <v>26.6</v>
+        <v>18.80904</v>
       </c>
       <c r="K69" s="8">
         <v>56993</v>
@@ -46683,7 +46683,7 @@
       </c>
       <c r="I70" s="1"/>
       <c r="J70" s="8">
-        <v>27</v>
+        <v>19.091883</v>
       </c>
       <c r="K70" s="8">
         <v>63672</v>
@@ -47706,7 +47706,7 @@
       </c>
       <c r="I101" s="1"/>
       <c r="J101" s="8">
-        <v>28</v>
+        <v>19.79899</v>
       </c>
       <c r="K101" s="8">
         <v>1382147</v>
@@ -47739,7 +47739,7 @@
       </c>
       <c r="I102" s="1"/>
       <c r="J102" s="8">
-        <v>28.4</v>
+        <v>20.081833</v>
       </c>
       <c r="K102" s="8">
         <v>1508751</v>
@@ -47772,7 +47772,7 @@
       </c>
       <c r="I103" s="1"/>
       <c r="J103" s="8">
-        <v>28.8</v>
+        <v>20.364675</v>
       </c>
       <c r="K103" s="8">
         <v>1645745</v>
@@ -47805,7 +47805,7 @@
       </c>
       <c r="I104" s="1"/>
       <c r="J104" s="8">
-        <v>29.2</v>
+        <v>20.647518</v>
       </c>
       <c r="K104" s="8">
         <v>1793862</v>
@@ -47838,7 +47838,7 @@
       </c>
       <c r="I105" s="1"/>
       <c r="J105" s="8">
-        <v>38</v>
+        <v>26.870058</v>
       </c>
       <c r="K105" s="8">
         <v>1953874</v>
@@ -47871,7 +47871,7 @@
       </c>
       <c r="I106" s="1"/>
       <c r="J106" s="8">
-        <v>38.45</v>
+        <v>27.188256</v>
       </c>
       <c r="K106" s="8">
         <v>2126596</v>
@@ -47904,7 +47904,7 @@
       </c>
       <c r="I107" s="1"/>
       <c r="J107" s="8">
-        <v>38.9</v>
+        <v>27.506454</v>
       </c>
       <c r="K107" s="8">
         <v>2312885</v>
@@ -47937,7 +47937,7 @@
       </c>
       <c r="I108" s="1"/>
       <c r="J108" s="8">
-        <v>39.35</v>
+        <v>27.824652</v>
       </c>
       <c r="K108" s="8">
         <v>2513643</v>
@@ -47970,7 +47970,7 @@
       </c>
       <c r="I109" s="1"/>
       <c r="J109" s="8">
-        <v>39.8</v>
+        <v>28.14285</v>
       </c>
       <c r="K109" s="8">
         <v>2729816</v>
@@ -48003,7 +48003,7 @@
       </c>
       <c r="I110" s="1"/>
       <c r="J110" s="8">
-        <v>40.25</v>
+        <v>28.461048</v>
       </c>
       <c r="K110" s="8">
         <v>2962396</v>
@@ -48036,7 +48036,7 @@
       </c>
       <c r="I111" s="1"/>
       <c r="J111" s="8">
-        <v>40.7</v>
+        <v>28.779246</v>
       </c>
       <c r="K111" s="8">
         <v>3212422</v>
@@ -48168,7 +48168,7 @@
       </c>
       <c r="I115" s="1"/>
       <c r="J115" s="8">
-        <v>38</v>
+        <v>12.016655</v>
       </c>
       <c r="K115" s="8">
         <v>4409435</v>
@@ -48201,7 +48201,7 @@
       </c>
       <c r="I116" s="1"/>
       <c r="J116" s="8">
-        <v>38.45</v>
+        <v>12.158958</v>
       </c>
       <c r="K116" s="8">
         <v>4763953</v>
@@ -48234,7 +48234,7 @@
       </c>
       <c r="I117" s="1"/>
       <c r="J117" s="8">
-        <v>38.9</v>
+        <v>12.30126</v>
       </c>
       <c r="K117" s="8">
         <v>5143163</v>
@@ -48267,7 +48267,7 @@
       </c>
       <c r="I118" s="1"/>
       <c r="J118" s="8">
-        <v>39.35</v>
+        <v>12.443563</v>
       </c>
       <c r="K118" s="8">
         <v>5548444</v>
@@ -48300,7 +48300,7 @@
       </c>
       <c r="I119" s="1"/>
       <c r="J119" s="8">
-        <v>39.8</v>
+        <v>12.585865</v>
       </c>
       <c r="K119" s="8">
         <v>5981222</v>
@@ -48333,7 +48333,7 @@
       </c>
       <c r="I120" s="1"/>
       <c r="J120" s="8">
-        <v>40.25</v>
+        <v>12.728168</v>
       </c>
       <c r="K120" s="8">
         <v>6442972</v>
@@ -48828,7 +48828,7 @@
       </c>
       <c r="I135" s="1"/>
       <c r="J135" s="8">
-        <v>41.7</v>
+        <v>29.486353</v>
       </c>
       <c r="K135" s="8">
         <v>17975355</v>
@@ -48861,7 +48861,7 @@
       </c>
       <c r="I136" s="1"/>
       <c r="J136" s="8">
-        <v>42.15</v>
+        <v>29.804551</v>
       </c>
       <c r="K136" s="8">
         <v>19132967</v>
@@ -48894,7 +48894,7 @@
       </c>
       <c r="I137" s="1"/>
       <c r="J137" s="8">
-        <v>42.6</v>
+        <v>30.122749</v>
       </c>
       <c r="K137" s="8">
         <v>20349823</v>
@@ -48927,7 +48927,7 @@
       </c>
       <c r="I138" s="1"/>
       <c r="J138" s="8">
-        <v>43.05</v>
+        <v>30.440947</v>
       </c>
       <c r="K138" s="8">
         <v>21627791</v>
@@ -48960,7 +48960,7 @@
       </c>
       <c r="I139" s="1"/>
       <c r="J139" s="8">
-        <v>43.5</v>
+        <v>30.759145</v>
       </c>
       <c r="K139" s="8">
         <v>22968714</v>
@@ -48993,7 +48993,7 @@
       </c>
       <c r="I140" s="1"/>
       <c r="J140" s="8">
-        <v>43.95</v>
+        <v>31.077343</v>
       </c>
       <c r="K140" s="8">
         <v>24374399</v>
@@ -49026,7 +49026,7 @@
       </c>
       <c r="I141" s="1"/>
       <c r="J141" s="8">
-        <v>44.4</v>
+        <v>31.395541</v>
       </c>
       <c r="K141" s="8">
         <v>25846612</v>
@@ -49356,7 +49356,7 @@
       </c>
       <c r="I151" s="1"/>
       <c r="J151" s="8">
-        <v>41.25</v>
+        <v>13.044395</v>
       </c>
       <c r="K151" s="8">
         <v>44568956</v>
@@ -49389,7 +49389,7 @@
       </c>
       <c r="I152" s="1"/>
       <c r="J152" s="8">
-        <v>41.7</v>
+        <v>13.186698</v>
       </c>
       <c r="K152" s="8">
         <v>46868714</v>
@@ -49422,7 +49422,7 @@
       </c>
       <c r="I153" s="1"/>
       <c r="J153" s="8">
-        <v>42.15</v>
+        <v>13.329</v>
       </c>
       <c r="K153" s="8">
         <v>49249644</v>
@@ -49455,7 +49455,7 @@
       </c>
       <c r="I154" s="1"/>
       <c r="J154" s="8">
-        <v>42.6</v>
+        <v>13.471303</v>
       </c>
       <c r="K154" s="8">
         <v>51712126</v>
@@ -49488,7 +49488,7 @@
       </c>
       <c r="I155" s="1"/>
       <c r="J155" s="8">
-        <v>51</v>
+        <v>16.127616</v>
       </c>
       <c r="K155" s="8">
         <v>54256362</v>
@@ -49521,7 +49521,7 @@
       </c>
       <c r="I156" s="1"/>
       <c r="J156" s="8">
-        <v>51.5</v>
+        <v>16.28573</v>
       </c>
       <c r="K156" s="8">
         <v>56882369</v>
@@ -49554,7 +49554,7 @@
       </c>
       <c r="I157" s="1"/>
       <c r="J157" s="8">
-        <v>52</v>
+        <v>16.443844</v>
       </c>
       <c r="K157" s="8">
         <v>59589969</v>
@@ -49587,7 +49587,7 @@
       </c>
       <c r="I158" s="1"/>
       <c r="J158" s="8">
-        <v>52.5</v>
+        <v>16.601958</v>
       </c>
       <c r="K158" s="8">
         <v>62378779</v>
@@ -49620,7 +49620,7 @@
       </c>
       <c r="I159" s="1"/>
       <c r="J159" s="8">
-        <v>53</v>
+        <v>16.760072</v>
       </c>
       <c r="K159" s="8">
         <v>65248202</v>
@@ -49653,7 +49653,7 @@
       </c>
       <c r="I160" s="1"/>
       <c r="J160" s="8">
-        <v>53.5</v>
+        <v>16.918185</v>
       </c>
       <c r="K160" s="8">
         <v>68197420</v>
@@ -49686,7 +49686,7 @@
       </c>
       <c r="I161" s="1"/>
       <c r="J161" s="8">
-        <v>54</v>
+        <v>17.076299</v>
       </c>
       <c r="K161" s="8">
         <v>71225385</v>
@@ -50478,7 +50478,7 @@
       </c>
       <c r="I185" s="1"/>
       <c r="J185" s="8">
-        <v>55</v>
+        <v>17.392527</v>
       </c>
       <c r="K185" s="8">
         <v>160328109</v>
@@ -50511,7 +50511,7 @@
       </c>
       <c r="I186" s="1"/>
       <c r="J186" s="8">
-        <v>55.5</v>
+        <v>17.550641</v>
       </c>
       <c r="K186" s="8">
         <v>164240114</v>
@@ -50544,7 +50544,7 @@
       </c>
       <c r="I187" s="1"/>
       <c r="J187" s="8">
-        <v>56</v>
+        <v>17.708755</v>
       </c>
       <c r="K187" s="8">
         <v>168116180</v>
@@ -50577,7 +50577,7 @@
       </c>
       <c r="I188" s="1"/>
       <c r="J188" s="8">
-        <v>56.5</v>
+        <v>17.866869</v>
       </c>
       <c r="K188" s="8">
         <v>171949228</v>
@@ -50610,7 +50610,7 @@
       </c>
       <c r="I189" s="1"/>
       <c r="J189" s="8">
-        <v>57</v>
+        <v>18.024983</v>
       </c>
       <c r="K189" s="8">
         <v>175732111</v>
@@ -50643,7 +50643,7 @@
       </c>
       <c r="I190" s="1"/>
       <c r="J190" s="8">
-        <v>57.5</v>
+        <v>18.183097</v>
       </c>
       <c r="K190" s="8">
         <v>179457631</v>
@@ -50676,7 +50676,7 @@
       </c>
       <c r="I191" s="1"/>
       <c r="J191" s="8">
-        <v>58</v>
+        <v>18.34121</v>
       </c>
       <c r="K191" s="8">
         <v>183118566</v>
@@ -50808,7 +50808,7 @@
       </c>
       <c r="I195" s="1"/>
       <c r="J195" s="8">
-        <v>51</v>
+        <v>36.062446</v>
       </c>
       <c r="K195" s="8">
         <v>198213423</v>
@@ -50841,7 +50841,7 @@
       </c>
       <c r="I196" s="1"/>
       <c r="J196" s="8">
-        <v>51.5</v>
+        <v>36.415999</v>
       </c>
       <c r="K196" s="8">
         <v>202177691</v>
@@ -50874,7 +50874,7 @@
       </c>
       <c r="I197" s="1"/>
       <c r="J197" s="8">
-        <v>52</v>
+        <v>36.769553</v>
       </c>
       <c r="K197" s="8">
         <v>206221244</v>
@@ -50907,7 +50907,7 @@
       </c>
       <c r="I198" s="1"/>
       <c r="J198" s="8">
-        <v>52.5</v>
+        <v>37.123106</v>
       </c>
       <c r="K198" s="8">
         <v>210345668</v>
@@ -50940,7 +50940,7 @@
       </c>
       <c r="I199" s="1"/>
       <c r="J199" s="8">
-        <v>53</v>
+        <v>37.476659</v>
       </c>
       <c r="K199" s="8">
         <v>214552581</v>
@@ -50973,7 +50973,7 @@
       </c>
       <c r="I200" s="1"/>
       <c r="J200" s="8">
-        <v>53.5</v>
+        <v>37.830213</v>
       </c>
       <c r="K200" s="8">
         <v>218843632</v>
@@ -51798,7 +51798,7 @@
       </c>
       <c r="I225" s="1"/>
       <c r="J225" s="8">
-        <v>64</v>
+        <v>45.254834</v>
       </c>
       <c r="K225" s="8">
         <v>359036159</v>
@@ -51831,7 +51831,7 @@
       </c>
       <c r="I226" s="1"/>
       <c r="J226" s="8">
-        <v>64.55</v>
+        <v>45.643743</v>
       </c>
       <c r="K226" s="8">
         <v>366216882</v>
@@ -51864,7 +51864,7 @@
       </c>
       <c r="I227" s="1"/>
       <c r="J227" s="8">
-        <v>65.1</v>
+        <v>46.032651</v>
       </c>
       <c r="K227" s="8">
         <v>373541219</v>
@@ -51897,7 +51897,7 @@
       </c>
       <c r="I228" s="1"/>
       <c r="J228" s="8">
-        <v>65.65</v>
+        <v>46.42156</v>
       </c>
       <c r="K228" s="8">
         <v>381012043</v>
@@ -51930,7 +51930,7 @@
       </c>
       <c r="I229" s="1"/>
       <c r="J229" s="8">
-        <v>66.2</v>
+        <v>46.810469</v>
       </c>
       <c r="K229" s="8">
         <v>388632283</v>
@@ -51963,7 +51963,7 @@
       </c>
       <c r="I230" s="1"/>
       <c r="J230" s="8">
-        <v>66.75</v>
+        <v>47.199378</v>
       </c>
       <c r="K230" s="8">
         <v>396404928</v>
@@ -52458,7 +52458,7 @@
       </c>
       <c r="I245" s="1"/>
       <c r="J245" s="8">
-        <v>64</v>
+        <v>20.238577</v>
       </c>
       <c r="K245" s="8">
         <v>533508831</v>
@@ -52491,7 +52491,7 @@
       </c>
       <c r="I246" s="1"/>
       <c r="J246" s="8">
-        <v>64.55</v>
+        <v>20.412502</v>
       </c>
       <c r="K246" s="8">
         <v>544179007</v>
@@ -52524,7 +52524,7 @@
       </c>
       <c r="I247" s="1"/>
       <c r="J247" s="8">
-        <v>65.1</v>
+        <v>20.586428</v>
       </c>
       <c r="K247" s="8">
         <v>555062587</v>
@@ -52557,7 +52557,7 @@
       </c>
       <c r="I248" s="1"/>
       <c r="J248" s="8">
-        <v>65.65</v>
+        <v>20.760353</v>
       </c>
       <c r="K248" s="8">
         <v>566163838</v>
@@ -52590,7 +52590,7 @@
       </c>
       <c r="I249" s="1"/>
       <c r="J249" s="8">
-        <v>66.2</v>
+        <v>20.934278</v>
       </c>
       <c r="K249" s="8">
         <v>577487114</v>
@@ -52623,7 +52623,7 @@
       </c>
       <c r="I250" s="1"/>
       <c r="J250" s="8">
-        <v>66.75</v>
+        <v>21.108203</v>
       </c>
       <c r="K250" s="8">
         <v>589036856</v>

</xml_diff>